<commit_message>
Balanceo con el MRP alineado y % a CABA en revendidos
Regenerado con el MRP que compra por la producción de los
Aprovechamientos: todos los checks en verde. La cascada de revendidos
aplica el % de unidades que van a CABA (tarjeta AGC), como el MRP.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E33CYXtZ2f33D1RjoRdR65
</commit_message>
<xml_diff>
--- a/salida/Balanceo_Materiales_y_Linea.xlsx
+++ b/salida/Balanceo_Materiales_y_Linea.xlsx
@@ -19862,15 +19862,15 @@
       </c>
       <c r="H8" s="17" t="n">
         <f aca="false">INDEX(Links!$C$17:$L$17,1,(Resumen!$C$3-2025))</f>
-        <v>7424.858444</v>
+        <v>7436.458444</v>
       </c>
       <c r="I8" s="6" t="str">
         <f aca="false">IF(ROUND(H8-D8,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J8" s="17" t="n">
         <f aca="false">H8-D8</f>
-        <v>-11.5999999999995</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19902,7 +19902,7 @@
       </c>
       <c r="H9" s="17" t="n">
         <f aca="false">INDEX(Links!$C$18:$L$18,1,(Resumen!$C$3-2025))</f>
-        <v>30860.7706862536</v>
+        <v>30814.97872</v>
       </c>
       <c r="I9" s="6" t="str">
         <f aca="false">IF(ROUND(H9-D9,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -19910,7 +19910,7 @@
       </c>
       <c r="J9" s="17" t="n">
         <f aca="false">H9-D9</f>
-        <v>45.7919662536006</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19942,15 +19942,15 @@
       </c>
       <c r="H10" s="17" t="n">
         <f aca="false">INDEX(Links!$C$19:$L$19,1,(Resumen!$C$3-2025))</f>
-        <v>1842.87697319699</v>
+        <v>1844.928079</v>
       </c>
       <c r="I10" s="6" t="str">
         <f aca="false">IF(ROUND(H10-D10,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J10" s="17" t="n">
         <f aca="false">H10-D10</f>
-        <v>-2.05110580300993</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20022,15 +20022,15 @@
       </c>
       <c r="H12" s="17" t="n">
         <f aca="false">INDEX(Links!$C$21:$L$21,1,(Resumen!$C$3-2025))</f>
-        <v>6669</v>
+        <v>6689.88</v>
       </c>
       <c r="I12" s="6" t="str">
         <f aca="false">IF(ROUND(H12-D12,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J12" s="17" t="n">
         <f aca="false">H12-D12</f>
-        <v>-20.8800000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20062,15 +20062,15 @@
       </c>
       <c r="H13" s="17" t="n">
         <f aca="false">INDEX(Links!$C$22:$L$22,1,(Resumen!$C$3-2025))</f>
-        <v>32915</v>
+        <v>33037.68</v>
       </c>
       <c r="I13" s="6" t="str">
         <f aca="false">IF(ROUND(H13-D13,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J13" s="17" t="n">
         <f aca="false">H13-D13</f>
-        <v>-122.68</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20102,15 +20102,15 @@
       </c>
       <c r="H14" s="17" t="n">
         <f aca="false">INDEX(Links!$C$23:$L$23,1,(Resumen!$C$3-2025))</f>
-        <v>2011</v>
+        <v>2018</v>
       </c>
       <c r="I14" s="6" t="str">
         <f aca="false">IF(ROUND(H14-D14,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J14" s="17" t="n">
         <f aca="false">H14-D14</f>
-        <v>-7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20142,15 +20142,15 @@
       </c>
       <c r="H15" s="17" t="n">
         <f aca="false">INDEX(Links!$C$24:$L$24,1,(Resumen!$C$3-2025))</f>
-        <v>453.2705332</v>
+        <v>453.6705332</v>
       </c>
       <c r="I15" s="6" t="str">
         <f aca="false">IF(ROUND(H15-D15,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J15" s="17" t="n">
         <f aca="false">H15-D15</f>
-        <v>-0.400000000000034</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20182,7 +20182,7 @@
       </c>
       <c r="H16" s="17" t="n">
         <f aca="false">INDEX(Links!$C$25:$L$25,1,(Resumen!$C$3-2025))</f>
-        <v>998.259982820404</v>
+        <v>997.9951731</v>
       </c>
       <c r="I16" s="6" t="str">
         <f aca="false">IF(ROUND(H16-D16,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -20190,7 +20190,7 @@
       </c>
       <c r="J16" s="17" t="n">
         <f aca="false">H16-D16</f>
-        <v>0.26480972040406</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20222,15 +20222,15 @@
       </c>
       <c r="H17" s="17" t="n">
         <f aca="false">INDEX(Links!$C$26:$L$26,1,(Resumen!$C$3-2025))</f>
-        <v>217.569856</v>
+        <v>217.809856</v>
       </c>
       <c r="I17" s="6" t="str">
         <f aca="false">IF(ROUND(H17-D17,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J17" s="17" t="n">
         <f aca="false">H17-D17</f>
-        <v>-0.240000000000009</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20262,7 +20262,7 @@
       </c>
       <c r="H18" s="17" t="n">
         <f aca="false">INDEX(Links!$C$27:$L$27,1,(Resumen!$C$3-2025))</f>
-        <v>145.176074484914</v>
+        <v>145.2065706</v>
       </c>
       <c r="I18" s="6" t="str">
         <f aca="false">IF(ROUND(H18-D18,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -20270,7 +20270,7 @@
       </c>
       <c r="J18" s="17" t="n">
         <f aca="false">H18-D18</f>
-        <v>-0.030496115085981</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20302,15 +20302,15 @@
       </c>
       <c r="H19" s="17" t="n">
         <f aca="false">INDEX(Links!$C$28:$L$28,1,(Resumen!$C$3-2025))</f>
-        <v>322</v>
+        <v>323.64</v>
       </c>
       <c r="I19" s="6" t="str">
         <f aca="false">IF(ROUND(H19-D19,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J19" s="17" t="n">
         <f aca="false">H19-D19</f>
-        <v>-1.63999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20342,15 +20342,15 @@
       </c>
       <c r="H20" s="17" t="n">
         <f aca="false">INDEX(Links!$C$29:$L$29,1,(Resumen!$C$3-2025))</f>
-        <v>708</v>
+        <v>710.44</v>
       </c>
       <c r="I20" s="6" t="str">
         <f aca="false">IF(ROUND(H20-D20,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J20" s="17" t="n">
         <f aca="false">H20-D20</f>
-        <v>-2.44000000000005</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20382,15 +20382,15 @@
       </c>
       <c r="H21" s="17" t="n">
         <f aca="false">INDEX(Links!$C$30:$L$30,1,(Resumen!$C$3-2025))</f>
-        <v>155</v>
+        <v>156.32</v>
       </c>
       <c r="I21" s="6" t="str">
         <f aca="false">IF(ROUND(H21-D21,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J21" s="17" t="n">
         <f aca="false">H21-D21</f>
-        <v>-1.31999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20422,15 +20422,15 @@
       </c>
       <c r="H22" s="17" t="n">
         <f aca="false">INDEX(Links!$C$31:$L$31,1,(Resumen!$C$3-2025))</f>
-        <v>102</v>
+        <v>102.24</v>
       </c>
       <c r="I22" s="6" t="str">
         <f aca="false">IF(ROUND(H22-D22,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J22" s="17" t="n">
         <f aca="false">H22-D22</f>
-        <v>-0.239999999999995</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20462,15 +20462,15 @@
       </c>
       <c r="H23" s="17" t="n">
         <f aca="false">INDEX(Links!$C$32:$L$32,1,(Resumen!$C$3-2025))</f>
-        <v>56487.4910822847</v>
+        <v>56575.8368575054</v>
       </c>
       <c r="I23" s="6" t="str">
         <f aca="false">IF(ROUND(H23-D23,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J23" s="17" t="n">
         <f aca="false">H23-D23</f>
-        <v>-88.3457752206959</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20502,15 +20502,15 @@
       </c>
       <c r="H24" s="17" t="n">
         <f aca="false">INDEX(Links!$C$33:$L$33,1,(Resumen!$C$3-2025))</f>
-        <v>4783.22920387376</v>
+        <v>4860.71011839089</v>
       </c>
       <c r="I24" s="6" t="str">
         <f aca="false">IF(ROUND(H24-D24,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J24" s="17" t="n">
         <f aca="false">H24-D24</f>
-        <v>-77.4809145171303</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20542,7 +20542,7 @@
       </c>
       <c r="H25" s="17" t="n">
         <f aca="false">INDEX(Links!$C$34:$L$34,1,(Resumen!$C$3-2025))</f>
-        <v>30068.838280126</v>
+        <v>29554.3203107948</v>
       </c>
       <c r="I25" s="6" t="str">
         <f aca="false">IF(ROUND(H25-D25,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -20550,7 +20550,7 @@
       </c>
       <c r="J25" s="17" t="n">
         <f aca="false">H25-D25</f>
-        <v>514.517969331202</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20582,15 +20582,15 @@
       </c>
       <c r="H26" s="17" t="n">
         <f aca="false">INDEX(Links!$C$35:$L$35,1,(Resumen!$C$3-2025))</f>
-        <v>1741.3814292141</v>
+        <v>1751.36955653994</v>
       </c>
       <c r="I26" s="6" t="str">
         <f aca="false">IF(ROUND(H26-D26,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J26" s="17" t="n">
         <f aca="false">H26-D26</f>
-        <v>-9.98812732583997</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20622,15 +20622,15 @@
       </c>
       <c r="H27" s="17" t="n">
         <f aca="false">INDEX(Links!$C$36:$L$36,1,(Resumen!$C$3-2025))</f>
-        <v>2458.50580352832</v>
+        <v>2471.83311933763</v>
       </c>
       <c r="I27" s="6" t="str">
         <f aca="false">IF(ROUND(H27-D27,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J27" s="17" t="n">
         <f aca="false">H27-D27</f>
-        <v>-13.3273158093098</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20662,15 +20662,15 @@
       </c>
       <c r="H28" s="17" t="n">
         <f aca="false">INDEX(Links!$C$37:$L$37,1,(Resumen!$C$3-2025))</f>
-        <v>466.916593765414</v>
+        <v>468.458588756731</v>
       </c>
       <c r="I28" s="6" t="str">
         <f aca="false">IF(ROUND(H28-D28,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J28" s="17" t="n">
         <f aca="false">H28-D28</f>
-        <v>-1.54199499131698</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20702,15 +20702,15 @@
       </c>
       <c r="H29" s="17" t="n">
         <f aca="false">INDEX(Links!$C$38:$L$38,1,(Resumen!$C$3-2025))</f>
-        <v>243.56826057903</v>
+        <v>244.066833405312</v>
       </c>
       <c r="I29" s="6" t="str">
         <f aca="false">IF(ROUND(H29-D29,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J29" s="17" t="n">
         <f aca="false">H29-D29</f>
-        <v>-0.498572826281986</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20742,15 +20742,15 @@
       </c>
       <c r="H30" s="17" t="n">
         <f aca="false">INDEX(Links!$C$39:$L$39,1,(Resumen!$C$3-2025))</f>
-        <v>140.865463166495</v>
+        <v>141.356355954645</v>
       </c>
       <c r="I30" s="6" t="str">
         <f aca="false">IF(ROUND(H30-D30,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J30" s="17" t="n">
         <f aca="false">H30-D30</f>
-        <v>-0.490892788150006</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20782,15 +20782,15 @@
       </c>
       <c r="H31" s="17" t="n">
         <f aca="false">INDEX(Links!$C$40:$L$40,1,(Resumen!$C$3-2025))</f>
-        <v>1212.31741440213</v>
+        <v>1218.24282190818</v>
       </c>
       <c r="I31" s="6" t="str">
         <f aca="false">IF(ROUND(H31-D31,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J31" s="17" t="n">
         <f aca="false">H31-D31</f>
-        <v>-5.92540750605008</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20822,15 +20822,15 @@
       </c>
       <c r="H32" s="17" t="n">
         <f aca="false">INDEX(Links!$C$41:$L$41,1,(Resumen!$C$3-2025))</f>
-        <v>6542.68065117681</v>
+        <v>6648.91332717417</v>
       </c>
       <c r="I32" s="6" t="str">
         <f aca="false">IF(ROUND(H32-D32,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J32" s="17" t="n">
         <f aca="false">H32-D32</f>
-        <v>-106.23267599736</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20862,7 +20862,7 @@
       </c>
       <c r="H33" s="17" t="n">
         <f aca="false">INDEX(Links!$C$42:$L$42,1,(Resumen!$C$3-2025))</f>
-        <v>2330.94823134952</v>
+        <v>2270.47576029921</v>
       </c>
       <c r="I33" s="6" t="str">
         <f aca="false">IF(ROUND(H33-D33,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -20870,7 +20870,7 @@
       </c>
       <c r="J33" s="17" t="n">
         <f aca="false">H33-D33</f>
-        <v>60.4724710503101</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20902,15 +20902,15 @@
       </c>
       <c r="H34" s="17" t="n">
         <f aca="false">INDEX(Links!$C$43:$L$43,1,(Resumen!$C$3-2025))</f>
-        <v>370.076373535804</v>
+        <v>372.61985757759</v>
       </c>
       <c r="I34" s="6" t="str">
         <f aca="false">IF(ROUND(H34-D34,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J34" s="17" t="n">
         <f aca="false">H34-D34</f>
-        <v>-2.54348404178597</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20942,15 +20942,15 @@
       </c>
       <c r="H35" s="17" t="n">
         <f aca="false">INDEX(Links!$C$44:$L$44,1,(Resumen!$C$3-2025))</f>
-        <v>127.111453828946</v>
+        <v>127.86907204172</v>
       </c>
       <c r="I35" s="6" t="str">
         <f aca="false">IF(ROUND(H35-D35,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J35" s="17" t="n">
         <f aca="false">H35-D35</f>
-        <v>-0.757618212774005</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20982,15 +20982,15 @@
       </c>
       <c r="H36" s="17" t="n">
         <f aca="false">INDEX(Links!$C$45:$L$45,1,(Resumen!$C$3-2025))</f>
-        <v>299.856087233694</v>
+        <v>305.325058646191</v>
       </c>
       <c r="I36" s="6" t="str">
         <f aca="false">IF(ROUND(H36-D36,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J36" s="17" t="n">
         <f aca="false">H36-D36</f>
-        <v>-5.46897141249701</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21022,15 +21022,15 @@
       </c>
       <c r="H37" s="17" t="n">
         <f aca="false">INDEX(Links!$C$46:$L$46,1,(Resumen!$C$3-2025))</f>
-        <v>670.043702304348</v>
+        <v>670.71512861809</v>
       </c>
       <c r="I37" s="6" t="str">
         <f aca="false">IF(ROUND(H37-D37,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J37" s="17" t="n">
         <f aca="false">H37-D37</f>
-        <v>-0.671426313742018</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21062,15 +21062,15 @@
       </c>
       <c r="H38" s="17" t="n">
         <f aca="false">INDEX(Links!$C$47:$L$47,1,(Resumen!$C$3-2025))</f>
-        <v>143.930921797349</v>
+        <v>147.156028161701</v>
       </c>
       <c r="I38" s="6" t="str">
         <f aca="false">IF(ROUND(H38-D38,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="J38" s="17" t="n">
         <f aca="false">H38-D38</f>
-        <v>-3.225106364352</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21102,7 +21102,7 @@
       </c>
       <c r="H39" s="17" t="n">
         <f aca="false">INDEX(Links!$C$48:$L$48,1,(Resumen!$C$3-2025))</f>
-        <v>98.5440255727726</v>
+        <v>98.1040185823099</v>
       </c>
       <c r="I39" s="6" t="str">
         <f aca="false">IF(ROUND(H39-D39,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -21110,7 +21110,7 @@
       </c>
       <c r="J39" s="17" t="n">
         <f aca="false">H39-D39</f>
-        <v>0.440006990462692</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21183,15 +21183,15 @@
       </c>
       <c r="H43" s="19" t="n">
         <f aca="false">SUMIF($A$7:$A$39,$A43,H$7:H$39)</f>
-        <v>284344.145233451</v>
+        <v>284462.564373</v>
       </c>
       <c r="I43" s="21" t="n">
         <f aca="false">COUNTIFS($A$7:$A$39,$A43,$I$7:$I$39,"✖ No")</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J43" s="19" t="n">
         <f aca="false">SUMIF($A$7:$A$39,$A43,J$7:J$39)</f>
-        <v>-118.419139549409</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21220,15 +21220,15 @@
       </c>
       <c r="H44" s="19" t="n">
         <f aca="false">SUMIF($A$7:$A$39,$A44,H$7:H$39)</f>
-        <v>3101.27644650532</v>
+        <v>3107.3221329</v>
       </c>
       <c r="I44" s="21" t="n">
         <f aca="false">COUNTIFS($A$7:$A$39,$A44,$I$7:$I$39,"✖ No")</f>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J44" s="19" t="n">
         <f aca="false">SUMIF($A$7:$A$39,$A44,J$7:J$39)</f>
-        <v>-6.04568639468199</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21257,15 +21257,15 @@
       </c>
       <c r="H45" s="19" t="n">
         <f aca="false">SUMIF($A$7:$A$39,$A45,H$7:H$39)</f>
-        <v>108186.304977739</v>
+        <v>107927.372813695</v>
       </c>
       <c r="I45" s="21" t="n">
         <f aca="false">COUNTIFS($A$7:$A$39,$A45,$I$7:$I$39,"✖ No")</f>
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="J45" s="19" t="n">
         <f aca="false">SUMIF($A$7:$A$39,$A45,J$7:J$39)</f>
-        <v>258.932164044689</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21523,43 +21523,43 @@
       </c>
       <c r="C53" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$C$16:$C$23-Links!$N$503:$N$510,1)&lt;0))</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D53" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$D$16:$D$23-Links!$N$514:$N$521,1)&lt;0))</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E53" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$E$16:$E$23-Links!$N$525:$N$532,1)&lt;0))</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F53" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$F$16:$F$23-Links!$N$536:$N$543,1)&lt;0))</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G53" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$G$16:$G$23-Links!$N$547:$N$554,1)&lt;0))</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H53" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$H$16:$H$23-Links!$N$558:$N$565,1)&lt;0))</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I53" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$I$16:$I$23-Links!$N$569:$N$576,1)&lt;0))</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J53" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$J$16:$J$23-Links!$N$580:$N$587,1)&lt;0))</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K53" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$K$16:$K$23-Links!$N$591:$N$598,1)&lt;0))</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L53" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$L$16:$L$23-Links!$N$602:$N$609,1)&lt;0))</f>
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21763,43 +21763,43 @@
       </c>
       <c r="C58" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$C$24:$C$31-Links!$N$1025:$N$1032,1)&lt;0))</f>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D58" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$D$24:$D$31-Links!$N$1036:$N$1043,1)&lt;0))</f>
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E58" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$E$24:$E$31-Links!$N$1047:$N$1054,1)&lt;0))</f>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F58" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$F$24:$F$31-Links!$N$1058:$N$1065,1)&lt;0))</f>
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G58" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$G$24:$G$31-Links!$N$1069:$N$1076,1)&lt;0))</f>
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="H58" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$H$24:$H$31-Links!$N$1080:$N$1087,1)&lt;0))</f>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I58" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$I$24:$I$31-Links!$N$1091:$N$1098,1)&lt;0))</f>
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J58" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$J$24:$J$31-Links!$N$1102:$N$1109,1)&lt;0))</f>
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K58" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$K$24:$K$31-Links!$N$1113:$N$1120,1)&lt;0))</f>
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L58" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$L$24:$L$31-Links!$N$1124:$N$1131,1)&lt;0))</f>
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22003,43 +22003,43 @@
       </c>
       <c r="C63" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$C$32:$C$48-Links!$N$1441:$N$1457,1)&lt;0))</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D63" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$D$32:$D$48-Links!$N$1473:$N$1489,1)&lt;0))</f>
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="E63" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$E$32:$E$48-Links!$N$1505:$N$1521,1)&lt;0))</f>
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F63" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$F$32:$F$48-Links!$N$1537:$N$1553,1)&lt;0))</f>
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="G63" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$G$32:$G$48-Links!$N$1569:$N$1585,1)&lt;0))</f>
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="H63" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$H$32:$H$48-Links!$N$1601:$N$1617,1)&lt;0))</f>
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="I63" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$I$32:$I$48-Links!$N$1633:$N$1649,1)&lt;0))</f>
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="J63" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$J$32:$J$48-Links!$N$1665:$N$1681,1)&lt;0))</f>
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="K63" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$K$32:$K$48-Links!$N$1697:$N$1713,1)&lt;0))</f>
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="L63" s="22" t="n">
         <f aca="false">SUMPRODUCT(--(ROUND(Links!$L$32:$L$48-Links!$N$1729:$N$1745,1)&lt;0))</f>
-        <v>14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22242,7 +22242,7 @@
         <v>CHECKS 2035
 Producción ≥ demanda: ✔
 Sobrestock: 0.1%
-MRP cubre la producción: ✖ 5 productos</v>
+MRP cubre la producción: ✔</v>
       </c>
       <c r="AM5" s="27"/>
       <c r="AN5" s="27"/>
@@ -22717,7 +22717,7 @@
         <v>CHECKS 2035
 Producción ≥ demanda: ✔
 Sobrestock: 0.2%
-MRP cubre la producción: ✖ 6 productos</v>
+MRP cubre la producción: ✔</v>
       </c>
       <c r="AM20" s="27"/>
       <c r="AN20" s="27"/>
@@ -23193,7 +23193,7 @@
         <v>CHECKS 2035
 Producción ≥ demanda: ✔
 Sobrestock: 0.7%
-MRP cubre la producción: ✖ 14 productos</v>
+MRP cubre la producción: ✔</v>
       </c>
       <c r="AM35" s="27"/>
       <c r="AN35" s="27"/>
@@ -30159,7 +30159,7 @@
       </c>
       <c r="G8" s="17" t="n">
         <f aca="false">INDEX(Links!$N$62:$W$62,1,(Resumen!$C$3-2025))</f>
-        <v>521.994757185185</v>
+        <v>523.197720148148</v>
       </c>
       <c r="H8" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$62:$M$62,$O$5:$V$5)*IF(Links!$E$62="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$62="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -30167,11 +30167,11 @@
       </c>
       <c r="I8" s="17" t="n">
         <f aca="false">G8-H8</f>
-        <v>-1.2029629629626</v>
+        <v>0</v>
       </c>
       <c r="J8" s="6" t="str">
         <f aca="false">IF(ROUND(G8-H8,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K8" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C8,Links!$B$218:$B$342,0)),1)</f>
@@ -30215,7 +30215,7 @@
       </c>
       <c r="G9" s="17" t="n">
         <f aca="false">INDEX(Links!$N$63:$W$63,1,(Resumen!$C$3-2025))</f>
-        <v>5314.6475571878</v>
+        <v>5321.05489333333</v>
       </c>
       <c r="H9" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$63:$M$63,$O$5:$V$5)*IF(Links!$E$63="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$63="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -30223,11 +30223,11 @@
       </c>
       <c r="I9" s="17" t="n">
         <f aca="false">G9-H9</f>
-        <v>-6.40733614553119</v>
+        <v>0</v>
       </c>
       <c r="J9" s="6" t="str">
         <f aca="false">IF(ROUND(G9-H9,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K9" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C9,Links!$B$218:$B$342,0)),1)</f>
@@ -30271,7 +30271,7 @@
       </c>
       <c r="G10" s="17" t="n">
         <f aca="false">INDEX(Links!$N$64:$W$64,1,(Resumen!$C$3-2025))</f>
-        <v>256.925131546466</v>
+        <v>257.5285386</v>
       </c>
       <c r="H10" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$64:$M$64,$O$5:$V$5)*IF(Links!$E$64="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$64="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -30279,11 +30279,11 @@
       </c>
       <c r="I10" s="17" t="n">
         <f aca="false">G10-H10</f>
-        <v>-0.603407053534113</v>
+        <v>0</v>
       </c>
       <c r="J10" s="6" t="str">
         <f aca="false">IF(ROUND(G10-H10,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K10" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C10,Links!$B$218:$B$342,0)),1)</f>
@@ -30439,7 +30439,7 @@
       </c>
       <c r="G13" s="17" t="n">
         <f aca="false">INDEX(Links!$N$67:$W$67,1,(Resumen!$C$3-2025))</f>
-        <v>3568.80740370326</v>
+        <v>3577.03189843144</v>
       </c>
       <c r="H13" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$67:$M$67,$O$5:$V$5)*IF(Links!$E$67="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$67="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -30447,11 +30447,11 @@
       </c>
       <c r="I13" s="17" t="n">
         <f aca="false">G13-H13</f>
-        <v>-8.2244947281788</v>
+        <v>0</v>
       </c>
       <c r="J13" s="6" t="str">
         <f aca="false">IF(ROUND(G13-H13,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K13" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C13,Links!$B$218:$B$342,0)),1)</f>
@@ -30495,7 +30495,7 @@
       </c>
       <c r="G14" s="17" t="n">
         <f aca="false">INDEX(Links!$N$68:$W$68,1,(Resumen!$C$3-2025))</f>
-        <v>2891.64354068509</v>
+        <v>2898.30747750371</v>
       </c>
       <c r="H14" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$68:$M$68,$O$5:$V$5)*IF(Links!$E$68="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$68="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -30503,11 +30503,11 @@
       </c>
       <c r="I14" s="17" t="n">
         <f aca="false">G14-H14</f>
-        <v>-6.66393681862019</v>
+        <v>0</v>
       </c>
       <c r="J14" s="6" t="str">
         <f aca="false">IF(ROUND(G14-H14,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K14" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C14,Links!$B$218:$B$342,0)),1)</f>
@@ -30551,7 +30551,7 @@
       </c>
       <c r="G15" s="17" t="n">
         <f aca="false">INDEX(Links!$N$69:$W$69,1,(Resumen!$C$3-2025))</f>
-        <v>32779.5634799705</v>
+        <v>32819.0825035106</v>
       </c>
       <c r="H15" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$69:$M$69,$O$5:$V$5)*IF(Links!$E$69="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$69="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -30559,11 +30559,11 @@
       </c>
       <c r="I15" s="17" t="n">
         <f aca="false">G15-H15</f>
-        <v>-39.5190235400805</v>
+        <v>0</v>
       </c>
       <c r="J15" s="6" t="str">
         <f aca="false">IF(ROUND(G15-H15,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K15" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C15,Links!$B$218:$B$342,0)),1)</f>
@@ -30607,7 +30607,7 @@
       </c>
       <c r="G16" s="17" t="n">
         <f aca="false">INDEX(Links!$N$70:$W$70,1,(Resumen!$C$3-2025))</f>
-        <v>24593.6650064639</v>
+        <v>24623.3151153472</v>
       </c>
       <c r="H16" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$70:$M$70,$O$5:$V$5)*IF(Links!$E$70="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$70="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -30615,11 +30615,11 @@
       </c>
       <c r="I16" s="17" t="n">
         <f aca="false">G16-H16</f>
-        <v>-29.6501088832883</v>
+        <v>0</v>
       </c>
       <c r="J16" s="6" t="str">
         <f aca="false">IF(ROUND(G16-H16,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K16" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C16,Links!$B$218:$B$342,0)),1)</f>
@@ -30663,7 +30663,7 @@
       </c>
       <c r="G17" s="17" t="n">
         <f aca="false">INDEX(Links!$N$71:$W$71,1,(Resumen!$C$3-2025))</f>
-        <v>2716.10807117145</v>
+        <v>2722.48704530466</v>
       </c>
       <c r="H17" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$71:$M$71,$O$5:$V$5)*IF(Links!$E$71="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$71="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -30671,11 +30671,11 @@
       </c>
       <c r="I17" s="17" t="n">
         <f aca="false">G17-H17</f>
-        <v>-6.37897413320889</v>
+        <v>0</v>
       </c>
       <c r="J17" s="6" t="str">
         <f aca="false">IF(ROUND(G17-H17,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K17" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C17,Links!$B$218:$B$342,0)),1)</f>
@@ -30719,7 +30719,7 @@
       </c>
       <c r="G18" s="17" t="n">
         <f aca="false">INDEX(Links!$N$72:$W$72,1,(Resumen!$C$3-2025))</f>
-        <v>2480.7406076469</v>
+        <v>2486.5668044523</v>
       </c>
       <c r="H18" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$72:$M$72,$O$5:$V$5)*IF(Links!$E$72="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$72="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -30727,11 +30727,11 @@
       </c>
       <c r="I18" s="17" t="n">
         <f aca="false">G18-H18</f>
-        <v>-5.82619680539983</v>
+        <v>0</v>
       </c>
       <c r="J18" s="6" t="str">
         <f aca="false">IF(ROUND(G18-H18,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K18" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C18,Links!$B$218:$B$342,0)),1)</f>
@@ -30831,7 +30831,7 @@
       </c>
       <c r="G20" s="17" t="n">
         <f aca="false">INDEX(Links!$N$74:$W$74,1,(Resumen!$C$3-2025))</f>
-        <v>81723.5061034506</v>
+        <v>81841.925243</v>
       </c>
       <c r="H20" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$74:$M$74,$O$5:$V$5)*IF(Links!$E$74="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$74="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -30839,11 +30839,11 @@
       </c>
       <c r="I20" s="17" t="n">
         <f aca="false">G20-H20</f>
-        <v>-118.419139549398</v>
+        <v>0</v>
       </c>
       <c r="J20" s="6" t="str">
         <f aca="false">IF(ROUND(G20-H20,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K20" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C20,Links!$B$218:$B$342,0)),1)</f>
@@ -30887,7 +30887,7 @@
       </c>
       <c r="G21" s="17" t="n">
         <f aca="false">INDEX(Links!$N$75:$W$75,1,(Resumen!$C$3-2025))</f>
-        <v>5985.81112149988</v>
+        <v>5990.03823683055</v>
       </c>
       <c r="H21" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$75:$M$75,$O$5:$V$5)*IF(Links!$E$75="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$75="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -30895,11 +30895,11 @@
       </c>
       <c r="I21" s="17" t="n">
         <f aca="false">G21-H21</f>
-        <v>-4.22711533067013</v>
+        <v>0</v>
       </c>
       <c r="J21" s="6" t="str">
         <f aca="false">IF(ROUND(G21-H21,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K21" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C21,Links!$B$218:$B$342,0)),1)</f>
@@ -30943,7 +30943,7 @@
       </c>
       <c r="G22" s="17" t="n">
         <f aca="false">INDEX(Links!$N$76:$W$76,1,(Resumen!$C$3-2025))</f>
-        <v>7393.13414849997</v>
+        <v>7398.35465882979</v>
       </c>
       <c r="H22" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$76:$M$76,$O$5:$V$5)*IF(Links!$E$76="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$76="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -30951,11 +30951,11 @@
       </c>
       <c r="I22" s="17" t="n">
         <f aca="false">G22-H22</f>
-        <v>-5.2205103298129</v>
+        <v>0</v>
       </c>
       <c r="J22" s="6" t="str">
         <f aca="false">IF(ROUND(G22-H22,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K22" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C22,Links!$B$218:$B$342,0)),1)</f>
@@ -31111,7 +31111,7 @@
       </c>
       <c r="G25" s="17" t="n">
         <f aca="false">INDEX(Links!$N$79:$W$79,1,(Resumen!$C$3-2025))</f>
-        <v>22747.5316186761</v>
+        <v>22757.00514984</v>
       </c>
       <c r="H25" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$79:$M$79,$O$5:$V$5)*IF(Links!$E$79="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$79="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -31119,11 +31119,11 @@
       </c>
       <c r="I25" s="17" t="n">
         <f aca="false">G25-H25</f>
-        <v>-9.47353116389786</v>
+        <v>0</v>
       </c>
       <c r="J25" s="6" t="str">
         <f aca="false">IF(ROUND(G25-H25,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K25" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C25,Links!$B$218:$B$342,0)),1)</f>
@@ -31167,7 +31167,7 @@
       </c>
       <c r="G26" s="17" t="n">
         <f aca="false">INDEX(Links!$N$80:$W$80,1,(Resumen!$C$3-2025))</f>
-        <v>3579.29598591396</v>
+        <v>3581.93537903661</v>
       </c>
       <c r="H26" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$80:$M$80,$O$5:$V$5)*IF(Links!$E$80="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$80="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -31175,11 +31175,11 @@
       </c>
       <c r="I26" s="17" t="n">
         <f aca="false">G26-H26</f>
-        <v>-2.63939312265029</v>
+        <v>0</v>
       </c>
       <c r="J26" s="6" t="str">
         <f aca="false">IF(ROUND(G26-H26,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K26" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C26,Links!$B$218:$B$342,0)),1)</f>
@@ -31223,7 +31223,7 @@
       </c>
       <c r="G27" s="17" t="n">
         <f aca="false">INDEX(Links!$N$81:$W$81,1,(Resumen!$C$3-2025))</f>
-        <v>230247.830430856</v>
+        <v>230062.40052855</v>
       </c>
       <c r="H27" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$81:$M$81,$O$5:$V$5)*IF(Links!$E$81="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$81="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -31231,7 +31231,7 @@
       </c>
       <c r="I27" s="17" t="n">
         <f aca="false">G27-H27</f>
-        <v>185.429902306001</v>
+        <v>0</v>
       </c>
       <c r="J27" s="6" t="str">
         <f aca="false">IF(ROUND(G27-H27,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -31279,7 +31279,7 @@
       </c>
       <c r="G28" s="17" t="n">
         <f aca="false">INDEX(Links!$N$82:$W$82,1,(Resumen!$C$3-2025))</f>
-        <v>1269.48875671279</v>
+        <v>1268.51569616287</v>
       </c>
       <c r="H28" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$82:$M$82,$O$5:$V$5)*IF(Links!$E$82="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$82="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -31287,7 +31287,7 @@
       </c>
       <c r="I28" s="17" t="n">
         <f aca="false">G28-H28</f>
-        <v>0.97306054992373</v>
+        <v>0</v>
       </c>
       <c r="J28" s="6" t="str">
         <f aca="false">IF(ROUND(G28-H28,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -31391,7 +31391,7 @@
       </c>
       <c r="G30" s="17" t="n">
         <f aca="false">INDEX(Links!$N$84:$W$84,1,(Resumen!$C$3-2025))</f>
-        <v>40128.5061034506</v>
+        <v>40096.365243</v>
       </c>
       <c r="H30" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$84:$M$84,$O$5:$V$5)*IF(Links!$E$84="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$84="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -31399,7 +31399,7 @@
       </c>
       <c r="I30" s="17" t="n">
         <f aca="false">G30-H30</f>
-        <v>32.1408604505996</v>
+        <v>0</v>
       </c>
       <c r="J30" s="6" t="str">
         <f aca="false">IF(ROUND(G30-H30,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -31447,7 +31447,7 @@
       </c>
       <c r="G31" s="17" t="n">
         <f aca="false">INDEX(Links!$N$85:$W$85,1,(Resumen!$C$3-2025))</f>
-        <v>72201.1452334506</v>
+        <v>72169.004373</v>
       </c>
       <c r="H31" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$85:$M$85,$O$5:$V$5)*IF(Links!$E$85="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$85="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -31455,7 +31455,7 @@
       </c>
       <c r="I31" s="17" t="n">
         <f aca="false">G31-H31</f>
-        <v>32.1408604505996</v>
+        <v>0</v>
       </c>
       <c r="J31" s="6" t="str">
         <f aca="false">IF(ROUND(G31-H31,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -31503,7 +31503,7 @@
       </c>
       <c r="G32" s="17" t="n">
         <f aca="false">INDEX(Links!$N$86:$W$86,1,(Resumen!$C$3-2025))</f>
-        <v>7424.858444</v>
+        <v>7436.458444</v>
       </c>
       <c r="H32" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$86:$M$86,$O$5:$V$5)*IF(Links!$E$86="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$86="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -31511,11 +31511,11 @@
       </c>
       <c r="I32" s="17" t="n">
         <f aca="false">G32-H32</f>
-        <v>-11.5999999999995</v>
+        <v>0</v>
       </c>
       <c r="J32" s="6" t="str">
         <f aca="false">IF(ROUND(G32-H32,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K32" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C32,Links!$B$218:$B$342,0)),1)</f>
@@ -31559,7 +31559,7 @@
       </c>
       <c r="G33" s="17" t="n">
         <f aca="false">INDEX(Links!$N$87:$W$87,1,(Resumen!$C$3-2025))</f>
-        <v>30860.7706862536</v>
+        <v>30814.97872</v>
       </c>
       <c r="H33" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$87:$M$87,$O$5:$V$5)*IF(Links!$E$87="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$87="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -31567,7 +31567,7 @@
       </c>
       <c r="I33" s="17" t="n">
         <f aca="false">G33-H33</f>
-        <v>45.7919662536006</v>
+        <v>0</v>
       </c>
       <c r="J33" s="6" t="str">
         <f aca="false">IF(ROUND(G33-H33,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -31615,7 +31615,7 @@
       </c>
       <c r="G34" s="17" t="n">
         <f aca="false">INDEX(Links!$N$88:$W$88,1,(Resumen!$C$3-2025))</f>
-        <v>1842.87697319699</v>
+        <v>1844.928079</v>
       </c>
       <c r="H34" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$88:$M$88,$O$5:$V$5)*IF(Links!$E$88="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$88="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -31623,11 +31623,11 @@
       </c>
       <c r="I34" s="17" t="n">
         <f aca="false">G34-H34</f>
-        <v>-2.05110580300993</v>
+        <v>0</v>
       </c>
       <c r="J34" s="6" t="str">
         <f aca="false">IF(ROUND(G34-H34,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K34" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C34,Links!$B$218:$B$342,0)),1)</f>
@@ -31727,7 +31727,7 @@
       </c>
       <c r="G36" s="17" t="n">
         <f aca="false">INDEX(Links!$N$90:$W$90,1,(Resumen!$C$3-2025))</f>
-        <v>7424.858444</v>
+        <v>7436.458444</v>
       </c>
       <c r="H36" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$90:$M$90,$O$5:$V$5)*IF(Links!$E$90="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$90="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -31735,11 +31735,11 @@
       </c>
       <c r="I36" s="17" t="n">
         <f aca="false">G36-H36</f>
-        <v>-11.5999999999995</v>
+        <v>0</v>
       </c>
       <c r="J36" s="6" t="str">
         <f aca="false">IF(ROUND(G36-H36,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K36" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C36,Links!$B$218:$B$342,0)),1)</f>
@@ -31783,7 +31783,7 @@
       </c>
       <c r="G37" s="17" t="n">
         <f aca="false">INDEX(Links!$N$91:$W$91,1,(Resumen!$C$3-2025))</f>
-        <v>30860.7706862536</v>
+        <v>30814.97872</v>
       </c>
       <c r="H37" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$91:$M$91,$O$5:$V$5)*IF(Links!$E$91="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$91="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -31791,7 +31791,7 @@
       </c>
       <c r="I37" s="17" t="n">
         <f aca="false">G37-H37</f>
-        <v>45.7919662536006</v>
+        <v>0</v>
       </c>
       <c r="J37" s="6" t="str">
         <f aca="false">IF(ROUND(G37-H37,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -31839,7 +31839,7 @@
       </c>
       <c r="G38" s="17" t="n">
         <f aca="false">INDEX(Links!$N$92:$W$92,1,(Resumen!$C$3-2025))</f>
-        <v>1842.87697319699</v>
+        <v>1844.928079</v>
       </c>
       <c r="H38" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$92:$M$92,$O$5:$V$5)*IF(Links!$E$92="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$92="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -31847,11 +31847,11 @@
       </c>
       <c r="I38" s="17" t="n">
         <f aca="false">G38-H38</f>
-        <v>-2.05110580300993</v>
+        <v>0</v>
       </c>
       <c r="J38" s="6" t="str">
         <f aca="false">IF(ROUND(G38-H38,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K38" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C38,Links!$B$218:$B$342,0)),1)</f>
@@ -31951,7 +31951,7 @@
       </c>
       <c r="G40" s="17" t="n">
         <f aca="false">INDEX(Links!$N$94:$W$94,1,(Resumen!$C$3-2025))</f>
-        <v>40128.5061034506</v>
+        <v>40096.365243</v>
       </c>
       <c r="H40" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$94:$M$94,$O$5:$V$5)*IF(Links!$E$94="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$94="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -31959,7 +31959,7 @@
       </c>
       <c r="I40" s="17" t="n">
         <f aca="false">G40-H40</f>
-        <v>32.1408604505996</v>
+        <v>0</v>
       </c>
       <c r="J40" s="6" t="str">
         <f aca="false">IF(ROUND(G40-H40,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -32007,7 +32007,7 @@
       </c>
       <c r="G41" s="17" t="n">
         <f aca="false">INDEX(Links!$N$95:$W$95,1,(Resumen!$C$3-2025))</f>
-        <v>7424.858444</v>
+        <v>7436.458444</v>
       </c>
       <c r="H41" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$95:$M$95,$O$5:$V$5)*IF(Links!$E$95="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$95="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -32015,11 +32015,11 @@
       </c>
       <c r="I41" s="17" t="n">
         <f aca="false">G41-H41</f>
-        <v>-11.5999999999995</v>
+        <v>0</v>
       </c>
       <c r="J41" s="6" t="str">
         <f aca="false">IF(ROUND(G41-H41,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K41" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C41,Links!$B$218:$B$342,0)),1)</f>
@@ -32063,7 +32063,7 @@
       </c>
       <c r="G42" s="17" t="n">
         <f aca="false">INDEX(Links!$N$96:$W$96,1,(Resumen!$C$3-2025))</f>
-        <v>30860.7706862536</v>
+        <v>30814.97872</v>
       </c>
       <c r="H42" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$96:$M$96,$O$5:$V$5)*IF(Links!$E$96="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$96="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -32071,7 +32071,7 @@
       </c>
       <c r="I42" s="17" t="n">
         <f aca="false">G42-H42</f>
-        <v>45.7919662536006</v>
+        <v>0</v>
       </c>
       <c r="J42" s="6" t="str">
         <f aca="false">IF(ROUND(G42-H42,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -32119,7 +32119,7 @@
       </c>
       <c r="G43" s="17" t="n">
         <f aca="false">INDEX(Links!$N$97:$W$97,1,(Resumen!$C$3-2025))</f>
-        <v>1842.87697319699</v>
+        <v>1844.928079</v>
       </c>
       <c r="H43" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$97:$M$97,$O$5:$V$5)*IF(Links!$E$97="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$97="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -32127,11 +32127,11 @@
       </c>
       <c r="I43" s="17" t="n">
         <f aca="false">G43-H43</f>
-        <v>-2.05110580300993</v>
+        <v>0</v>
       </c>
       <c r="J43" s="6" t="str">
         <f aca="false">IF(ROUND(G43-H43,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K43" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C43,Links!$B$218:$B$342,0)),1)</f>
@@ -32231,7 +32231,7 @@
       </c>
       <c r="G45" s="17" t="n">
         <f aca="false">INDEX(Links!$N$99:$W$99,1,(Resumen!$C$3-2025))</f>
-        <v>80257.0122069013</v>
+        <v>80192.730486</v>
       </c>
       <c r="H45" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$99:$M$99,$O$5:$V$5)*IF(Links!$E$99="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$99="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -32239,7 +32239,7 @@
       </c>
       <c r="I45" s="17" t="n">
         <f aca="false">G45-H45</f>
-        <v>64.281720901301</v>
+        <v>0</v>
       </c>
       <c r="J45" s="6" t="str">
         <f aca="false">IF(ROUND(G45-H45,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -32343,7 +32343,7 @@
       </c>
       <c r="G47" s="17" t="n">
         <f aca="false">INDEX(Links!$N$101:$W$101,1,(Resumen!$C$3-2025))</f>
-        <v>7424.858444</v>
+        <v>7436.458444</v>
       </c>
       <c r="H47" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$101:$M$101,$O$5:$V$5)*IF(Links!$E$101="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$101="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -32351,11 +32351,11 @@
       </c>
       <c r="I47" s="17" t="n">
         <f aca="false">G47-H47</f>
-        <v>-11.5999999999995</v>
+        <v>0</v>
       </c>
       <c r="J47" s="6" t="str">
         <f aca="false">IF(ROUND(G47-H47,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K47" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C47,Links!$B$218:$B$342,0)),1)</f>
@@ -32399,7 +32399,7 @@
       </c>
       <c r="G48" s="17" t="n">
         <f aca="false">INDEX(Links!$N$102:$W$102,1,(Resumen!$C$3-2025))</f>
-        <v>30860.7706862536</v>
+        <v>30814.97872</v>
       </c>
       <c r="H48" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$102:$M$102,$O$5:$V$5)*IF(Links!$E$102="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$102="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -32407,7 +32407,7 @@
       </c>
       <c r="I48" s="17" t="n">
         <f aca="false">G48-H48</f>
-        <v>45.7919662536006</v>
+        <v>0</v>
       </c>
       <c r="J48" s="6" t="str">
         <f aca="false">IF(ROUND(G48-H48,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -32455,7 +32455,7 @@
       </c>
       <c r="G49" s="17" t="n">
         <f aca="false">INDEX(Links!$N$103:$W$103,1,(Resumen!$C$3-2025))</f>
-        <v>1842.87697319699</v>
+        <v>1844.928079</v>
       </c>
       <c r="H49" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$103:$M$103,$O$5:$V$5)*IF(Links!$E$103="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$103="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -32463,11 +32463,11 @@
       </c>
       <c r="I49" s="17" t="n">
         <f aca="false">G49-H49</f>
-        <v>-2.05110580300993</v>
+        <v>0</v>
       </c>
       <c r="J49" s="6" t="str">
         <f aca="false">IF(ROUND(G49-H49,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K49" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C49,Links!$B$218:$B$342,0)),1)</f>
@@ -32511,7 +32511,7 @@
       </c>
       <c r="G50" s="17" t="n">
         <f aca="false">INDEX(Links!$N$104:$W$104,1,(Resumen!$C$3-2025))</f>
-        <v>55146.1396445977</v>
+        <v>55121.5909428703</v>
       </c>
       <c r="H50" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$104:$M$104,$O$5:$V$5)*IF(Links!$E$104="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$104="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -32519,7 +32519,7 @@
       </c>
       <c r="I50" s="17" t="n">
         <f aca="false">G50-H50</f>
-        <v>24.5487017273626</v>
+        <v>0</v>
       </c>
       <c r="J50" s="6" t="str">
         <f aca="false">IF(ROUND(G50-H50,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -32567,7 +32567,7 @@
       </c>
       <c r="G51" s="17" t="n">
         <f aca="false">INDEX(Links!$N$105:$W$105,1,(Resumen!$C$3-2025))</f>
-        <v>72201.1452334506</v>
+        <v>72169.004373</v>
       </c>
       <c r="H51" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$105:$M$105,$O$5:$V$5)*IF(Links!$E$105="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$105="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -32575,7 +32575,7 @@
       </c>
       <c r="I51" s="17" t="n">
         <f aca="false">G51-H51</f>
-        <v>32.1408604505996</v>
+        <v>0</v>
       </c>
       <c r="J51" s="6" t="str">
         <f aca="false">IF(ROUND(G51-H51,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -32623,7 +32623,7 @@
       </c>
       <c r="G52" s="17" t="n">
         <f aca="false">INDEX(Links!$N$106:$W$106,1,(Resumen!$C$3-2025))</f>
-        <v>9478.96177621284</v>
+        <v>9471.36961748954</v>
       </c>
       <c r="H52" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$106:$M$106,$O$5:$V$5)*IF(Links!$E$106="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$106="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -32631,7 +32631,7 @@
       </c>
       <c r="I52" s="17" t="n">
         <f aca="false">G52-H52</f>
-        <v>7.59215872328969</v>
+        <v>0</v>
       </c>
       <c r="J52" s="6" t="str">
         <f aca="false">IF(ROUND(G52-H52,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -32679,7 +32679,7 @@
       </c>
       <c r="G53" s="17" t="n">
         <f aca="false">INDEX(Links!$N$107:$W$107,1,(Resumen!$C$3-2025))</f>
-        <v>72201.1452334506</v>
+        <v>72169.004373</v>
       </c>
       <c r="H53" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$107:$M$107,$O$5:$V$5)*IF(Links!$E$107="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$107="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -32687,7 +32687,7 @@
       </c>
       <c r="I53" s="17" t="n">
         <f aca="false">G53-H53</f>
-        <v>32.1408604505996</v>
+        <v>0</v>
       </c>
       <c r="J53" s="6" t="str">
         <f aca="false">IF(ROUND(G53-H53,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -32735,7 +32735,7 @@
       </c>
       <c r="G54" s="17" t="n">
         <f aca="false">INDEX(Links!$N$108:$W$108,1,(Resumen!$C$3-2025))</f>
-        <v>72201.1452334506</v>
+        <v>72169.004373</v>
       </c>
       <c r="H54" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$108:$M$108,$O$5:$V$5)*IF(Links!$E$108="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$108="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -32743,7 +32743,7 @@
       </c>
       <c r="I54" s="17" t="n">
         <f aca="false">G54-H54</f>
-        <v>32.1408604505996</v>
+        <v>0</v>
       </c>
       <c r="J54" s="6" t="str">
         <f aca="false">IF(ROUND(G54-H54,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -32791,7 +32791,7 @@
       </c>
       <c r="G55" s="17" t="n">
         <f aca="false">INDEX(Links!$N$109:$W$109,1,(Resumen!$C$3-2025))</f>
-        <v>72201.1452334506</v>
+        <v>72169.004373</v>
       </c>
       <c r="H55" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$109:$M$109,$O$5:$V$5)*IF(Links!$E$109="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$109="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -32799,7 +32799,7 @@
       </c>
       <c r="I55" s="17" t="n">
         <f aca="false">G55-H55</f>
-        <v>32.1408604505996</v>
+        <v>0</v>
       </c>
       <c r="J55" s="6" t="str">
         <f aca="false">IF(ROUND(G55-H55,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -32847,7 +32847,7 @@
       </c>
       <c r="G56" s="17" t="n">
         <f aca="false">INDEX(Links!$N$110:$W$110,1,(Resumen!$C$3-2025))</f>
-        <v>212143</v>
+        <v>212293.56</v>
       </c>
       <c r="H56" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$110:$M$110,$O$5:$V$5)*IF(Links!$E$110="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$110="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -32855,11 +32855,11 @@
       </c>
       <c r="I56" s="17" t="n">
         <f aca="false">G56-H56</f>
-        <v>-150.559999999998</v>
+        <v>0</v>
       </c>
       <c r="J56" s="6" t="str">
         <f aca="false">IF(ROUND(G56-H56,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K56" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C56,Links!$B$218:$B$342,0)),1)</f>
@@ -32959,7 +32959,7 @@
       </c>
       <c r="G58" s="17" t="n">
         <f aca="false">INDEX(Links!$N$112:$W$112,1,(Resumen!$C$3-2025))</f>
-        <v>41595</v>
+        <v>41745.56</v>
       </c>
       <c r="H58" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$112:$M$112,$O$5:$V$5)*IF(Links!$E$112="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$112="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -32967,11 +32967,11 @@
       </c>
       <c r="I58" s="17" t="n">
         <f aca="false">G58-H58</f>
-        <v>-150.559999999998</v>
+        <v>0</v>
       </c>
       <c r="J58" s="6" t="str">
         <f aca="false">IF(ROUND(G58-H58,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K58" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C58,Links!$B$218:$B$342,0)),1)</f>
@@ -33015,7 +33015,7 @@
       </c>
       <c r="G59" s="17" t="n">
         <f aca="false">INDEX(Links!$N$113:$W$113,1,(Resumen!$C$3-2025))</f>
-        <v>212143</v>
+        <v>212293.56</v>
       </c>
       <c r="H59" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$113:$M$113,$O$5:$V$5)*IF(Links!$E$113="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$113="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -33023,11 +33023,11 @@
       </c>
       <c r="I59" s="17" t="n">
         <f aca="false">G59-H59</f>
-        <v>-150.559999999998</v>
+        <v>0</v>
       </c>
       <c r="J59" s="6" t="str">
         <f aca="false">IF(ROUND(G59-H59,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K59" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C59,Links!$B$218:$B$342,0)),1)</f>
@@ -33127,7 +33127,7 @@
       </c>
       <c r="G61" s="17" t="n">
         <f aca="false">INDEX(Links!$N$115:$W$115,1,(Resumen!$C$3-2025))</f>
-        <v>14093.858444</v>
+        <v>14126.338444</v>
       </c>
       <c r="H61" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$115:$M$115,$O$5:$V$5)*IF(Links!$E$115="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$115="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -33135,11 +33135,11 @@
       </c>
       <c r="I61" s="17" t="n">
         <f aca="false">G61-H61</f>
-        <v>-32.4800000000014</v>
+        <v>0</v>
       </c>
       <c r="J61" s="6" t="str">
         <f aca="false">IF(ROUND(G61-H61,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K61" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C61,Links!$B$218:$B$342,0)),1)</f>
@@ -33183,7 +33183,7 @@
       </c>
       <c r="G62" s="17" t="n">
         <f aca="false">INDEX(Links!$N$116:$W$116,1,(Resumen!$C$3-2025))</f>
-        <v>63775.7706862536</v>
+        <v>63852.65872</v>
       </c>
       <c r="H62" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$116:$M$116,$O$5:$V$5)*IF(Links!$E$116="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$116="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -33191,11 +33191,11 @@
       </c>
       <c r="I62" s="17" t="n">
         <f aca="false">G62-H62</f>
-        <v>-76.8880337463997</v>
+        <v>0</v>
       </c>
       <c r="J62" s="6" t="str">
         <f aca="false">IF(ROUND(G62-H62,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K62" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C62,Links!$B$218:$B$342,0)),1)</f>
@@ -33239,7 +33239,7 @@
       </c>
       <c r="G63" s="17" t="n">
         <f aca="false">INDEX(Links!$N$117:$W$117,1,(Resumen!$C$3-2025))</f>
-        <v>3853.87697319699</v>
+        <v>3862.928079</v>
       </c>
       <c r="H63" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$117:$M$117,$O$5:$V$5)*IF(Links!$E$117="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$117="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -33247,11 +33247,11 @@
       </c>
       <c r="I63" s="17" t="n">
         <f aca="false">G63-H63</f>
-        <v>-9.05110580301016</v>
+        <v>0</v>
       </c>
       <c r="J63" s="6" t="str">
         <f aca="false">IF(ROUND(G63-H63,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K63" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C63,Links!$B$218:$B$342,0)),1)</f>
@@ -33295,7 +33295,7 @@
       </c>
       <c r="G64" s="17" t="n">
         <f aca="false">INDEX(Links!$N$118:$W$118,1,(Resumen!$C$3-2025))</f>
-        <v>284344.145233451</v>
+        <v>284462.564373</v>
       </c>
       <c r="H64" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$118:$M$118,$O$5:$V$5)*IF(Links!$E$118="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$118="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -33303,11 +33303,11 @@
       </c>
       <c r="I64" s="17" t="n">
         <f aca="false">G64-H64</f>
-        <v>-118.41913954902</v>
+        <v>0</v>
       </c>
       <c r="J64" s="6" t="str">
         <f aca="false">IF(ROUND(G64-H64,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K64" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C64,Links!$B$218:$B$342,0)),1)</f>
@@ -33351,7 +33351,7 @@
       </c>
       <c r="G65" s="17" t="n">
         <f aca="false">INDEX(Links!$N$119:$W$119,1,(Resumen!$C$3-2025))</f>
-        <v>1395.91255838675</v>
+        <v>1397.18763853586</v>
       </c>
       <c r="H65" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$119:$M$119,$O$5:$V$5)*IF(Links!$E$119="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$119="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -33359,11 +33359,11 @@
       </c>
       <c r="I65" s="17" t="n">
         <f aca="false">G65-H65</f>
-        <v>-1.27508014911064</v>
+        <v>0</v>
       </c>
       <c r="J65" s="6" t="str">
         <f aca="false">IF(ROUND(G65-H65,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K65" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C65,Links!$B$218:$B$342,0)),1)</f>
@@ -33407,7 +33407,7 @@
       </c>
       <c r="G66" s="17" t="n">
         <f aca="false">INDEX(Links!$N$120:$W$120,1,(Resumen!$C$3-2025))</f>
-        <v>1395.91255838675</v>
+        <v>1397.18763853586</v>
       </c>
       <c r="H66" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$120:$M$120,$O$5:$V$5)*IF(Links!$E$120="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$120="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -33415,11 +33415,11 @@
       </c>
       <c r="I66" s="17" t="n">
         <f aca="false">G66-H66</f>
-        <v>-1.27508014911064</v>
+        <v>0</v>
       </c>
       <c r="J66" s="6" t="str">
         <f aca="false">IF(ROUND(G66-H66,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K66" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C66,Links!$B$218:$B$342,0)),1)</f>
@@ -33565,7 +33565,7 @@
       </c>
       <c r="G71" s="17" t="n">
         <f aca="false">INDEX(Links!$N$123:$W$123,1,(Resumen!$C$3-2025))</f>
-        <v>348.982541570067</v>
+        <v>349.515073283333</v>
       </c>
       <c r="H71" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$123:$M$123,$O$69:$V$69)*IF(Links!$E$123="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$123="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -33573,11 +33573,11 @@
       </c>
       <c r="I71" s="17" t="n">
         <f aca="false">G71-H71</f>
-        <v>-0.532531713266906</v>
+        <v>0</v>
       </c>
       <c r="J71" s="6" t="str">
         <f aca="false">IF(ROUND(G71-H71,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K71" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C71,Links!$B$218:$B$342,0)),1)</f>
@@ -33621,7 +33621,7 @@
       </c>
       <c r="G72" s="17" t="n">
         <f aca="false">INDEX(Links!$N$124:$W$124,1,(Resumen!$C$3-2025))</f>
-        <v>165.185326161638</v>
+        <v>165.6221582</v>
       </c>
       <c r="H72" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$124:$M$124,$O$69:$V$69)*IF(Links!$E$124="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$124="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -33629,11 +33629,11 @@
       </c>
       <c r="I72" s="17" t="n">
         <f aca="false">G72-H72</f>
-        <v>-0.436832038361814</v>
+        <v>0</v>
       </c>
       <c r="J72" s="6" t="str">
         <f aca="false">IF(ROUND(G72-H72,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K72" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C72,Links!$B$218:$B$342,0)),1)</f>
@@ -33677,7 +33677,7 @@
       </c>
       <c r="G73" s="17" t="n">
         <f aca="false">INDEX(Links!$N$125:$W$125,1,(Resumen!$C$3-2025))</f>
-        <v>1550.5410664</v>
+        <v>1554.6210664</v>
       </c>
       <c r="H73" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$125:$M$125,$O$69:$V$69)*IF(Links!$E$125="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$125="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -33685,11 +33685,11 @@
       </c>
       <c r="I73" s="17" t="n">
         <f aca="false">G73-H73</f>
-        <v>-4.07999999999993</v>
+        <v>0</v>
       </c>
       <c r="J73" s="6" t="str">
         <f aca="false">IF(ROUND(G73-H73,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K73" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C73,Links!$B$218:$B$342,0)),1)</f>
@@ -33733,7 +33733,7 @@
       </c>
       <c r="G74" s="17" t="n">
         <f aca="false">INDEX(Links!$N$126:$W$126,1,(Resumen!$C$3-2025))</f>
-        <v>3412.51996564081</v>
+        <v>3416.8703462</v>
       </c>
       <c r="H74" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$126:$M$126,$O$69:$V$69)*IF(Links!$E$126="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$126="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -33741,11 +33741,11 @@
       </c>
       <c r="I74" s="17" t="n">
         <f aca="false">G74-H74</f>
-        <v>-4.3503805591904</v>
+        <v>0</v>
       </c>
       <c r="J74" s="6" t="str">
         <f aca="false">IF(ROUND(G74-H74,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K74" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C74,Links!$B$218:$B$342,0)),1)</f>
@@ -33789,7 +33789,7 @@
       </c>
       <c r="G75" s="17" t="n">
         <f aca="false">INDEX(Links!$N$127:$W$127,1,(Resumen!$C$3-2025))</f>
-        <v>1239.49186096983</v>
+        <v>1243.1528532</v>
       </c>
       <c r="H75" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$127:$M$127,$O$69:$V$69)*IF(Links!$E$127="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$127="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -33797,11 +33797,11 @@
       </c>
       <c r="I75" s="17" t="n">
         <f aca="false">G75-H75</f>
-        <v>-3.66099223017</v>
+        <v>0</v>
       </c>
       <c r="J75" s="6" t="str">
         <f aca="false">IF(ROUND(G75-H75,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K75" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C75,Links!$B$218:$B$342,0)),1)</f>
@@ -33845,7 +33845,7 @@
       </c>
       <c r="G76" s="17" t="n">
         <f aca="false">INDEX(Links!$N$128:$W$128,1,(Resumen!$C$3-2025))</f>
-        <v>2481.5305160204</v>
+        <v>2485.7457063</v>
       </c>
       <c r="H76" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$128:$M$128,$O$69:$V$69)*IF(Links!$E$128="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$128="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -33853,11 +33853,11 @@
       </c>
       <c r="I76" s="17" t="n">
         <f aca="false">G76-H76</f>
-        <v>-4.21519027960039</v>
+        <v>0</v>
       </c>
       <c r="J76" s="6" t="str">
         <f aca="false">IF(ROUND(G76-H76,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K76" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C76,Links!$B$218:$B$342,0)),1)</f>
@@ -33901,7 +33901,7 @@
       </c>
       <c r="G77" s="17" t="n">
         <f aca="false">INDEX(Links!$N$129:$W$129,1,(Resumen!$C$3-2025))</f>
-        <v>619.745930484914</v>
+        <v>621.5764266</v>
       </c>
       <c r="H77" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$129:$M$129,$O$69:$V$69)*IF(Links!$E$129="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$129="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -33909,11 +33909,11 @@
       </c>
       <c r="I77" s="17" t="n">
         <f aca="false">G77-H77</f>
-        <v>-1.83049611508602</v>
+        <v>0</v>
       </c>
       <c r="J77" s="6" t="str">
         <f aca="false">IF(ROUND(G77-H77,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K77" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C77,Links!$B$218:$B$342,0)),1)</f>
@@ -33957,7 +33957,7 @@
       </c>
       <c r="G78" s="17" t="n">
         <f aca="false">INDEX(Links!$N$130:$W$130,1,(Resumen!$C$3-2025))</f>
-        <v>510.050621038391</v>
+        <v>510.181354029263</v>
       </c>
       <c r="H78" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$130:$M$130,$O$69:$V$69)*IF(Links!$E$130="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$130="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -33965,11 +33965,11 @@
       </c>
       <c r="I78" s="17" t="n">
         <f aca="false">G78-H78</f>
-        <v>-0.130732990872502</v>
+        <v>0</v>
       </c>
       <c r="J78" s="6" t="str">
         <f aca="false">IF(ROUND(G78-H78,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K78" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C78,Links!$B$218:$B$342,0)),1)</f>
@@ -34013,7 +34013,7 @@
       </c>
       <c r="G79" s="17" t="n">
         <f aca="false">INDEX(Links!$N$131:$W$131,1,(Resumen!$C$3-2025))</f>
-        <v>89.6168013594519</v>
+        <v>89.620950951193</v>
       </c>
       <c r="H79" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$131:$M$131,$O$69:$V$69)*IF(Links!$E$131="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$131="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -34021,7 +34021,7 @@
       </c>
       <c r="I79" s="17" t="n">
         <f aca="false">G79-H79</f>
-        <v>-0.00414959174105434</v>
+        <v>0</v>
       </c>
       <c r="J79" s="6" t="str">
         <f aca="false">IF(ROUND(G79-H79,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -34069,7 +34069,7 @@
       </c>
       <c r="G80" s="17" t="n">
         <f aca="false">INDEX(Links!$N$132:$W$132,1,(Resumen!$C$3-2025))</f>
-        <v>56.65881665</v>
+        <v>56.70881665</v>
       </c>
       <c r="H80" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$132:$M$132,$O$69:$V$69)*IF(Links!$E$132="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$132="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -34077,11 +34077,11 @@
       </c>
       <c r="I80" s="17" t="n">
         <f aca="false">G80-H80</f>
-        <v>-0.0500000000000043</v>
+        <v>0</v>
       </c>
       <c r="J80" s="6" t="str">
         <f aca="false">IF(ROUND(G80-H80,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K80" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C80,Links!$B$218:$B$342,0)),1)</f>
@@ -34125,7 +34125,7 @@
       </c>
       <c r="G81" s="17" t="n">
         <f aca="false">INDEX(Links!$N$133:$W$133,1,(Resumen!$C$3-2025))</f>
-        <v>127.025500577619</v>
+        <v>127.028476578182</v>
       </c>
       <c r="H81" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$133:$M$133,$O$69:$V$69)*IF(Links!$E$133="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$133="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -34133,7 +34133,7 @@
       </c>
       <c r="I81" s="17" t="n">
         <f aca="false">G81-H81</f>
-        <v>-0.00297600056281055</v>
+        <v>0</v>
       </c>
       <c r="J81" s="6" t="str">
         <f aca="false">IF(ROUND(G81-H81,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -34181,7 +34181,7 @@
       </c>
       <c r="G82" s="17" t="n">
         <f aca="false">INDEX(Links!$N$134:$W$134,1,(Resumen!$C$3-2025))</f>
-        <v>1388.19529361605</v>
+        <v>1390.59738886517</v>
       </c>
       <c r="H82" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$134:$M$134,$O$69:$V$69)*IF(Links!$E$134="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$134="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -34189,11 +34189,11 @@
       </c>
       <c r="I82" s="17" t="n">
         <f aca="false">G82-H82</f>
-        <v>-2.40209524911984</v>
+        <v>0</v>
       </c>
       <c r="J82" s="6" t="str">
         <f aca="false">IF(ROUND(G82-H82,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K82" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C82,Links!$B$218:$B$342,0)),1)</f>
@@ -34237,7 +34237,7 @@
       </c>
       <c r="G83" s="17" t="n">
         <f aca="false">INDEX(Links!$N$135:$W$135,1,(Resumen!$C$3-2025))</f>
-        <v>560.468514400998</v>
+        <v>561.28410562221</v>
       </c>
       <c r="H83" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$135:$M$135,$O$69:$V$69)*IF(Links!$E$135="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$135="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -34245,11 +34245,11 @@
       </c>
       <c r="I83" s="17" t="n">
         <f aca="false">G83-H83</f>
-        <v>-0.815591221212003</v>
+        <v>0</v>
       </c>
       <c r="J83" s="6" t="str">
         <f aca="false">IF(ROUND(G83-H83,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K83" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C83,Links!$B$218:$B$342,0)),1)</f>
@@ -34293,7 +34293,7 @@
       </c>
       <c r="G84" s="17" t="n">
         <f aca="false">INDEX(Links!$N$136:$W$136,1,(Resumen!$C$3-2025))</f>
-        <v>27.2141466975798</v>
+        <v>27.2202319935</v>
       </c>
       <c r="H84" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$136:$M$136,$O$69:$V$69)*IF(Links!$E$136="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$136="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -34301,7 +34301,7 @@
       </c>
       <c r="I84" s="17" t="n">
         <f aca="false">G84-H84</f>
-        <v>-0.00608529592020091</v>
+        <v>0</v>
       </c>
       <c r="J84" s="6" t="str">
         <f aca="false">IF(ROUND(G84-H84,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -34349,7 +34349,7 @@
       </c>
       <c r="G85" s="17" t="n">
         <f aca="false">INDEX(Links!$N$137:$W$137,1,(Resumen!$C$3-2025))</f>
-        <v>99.5846800800629</v>
+        <v>99.75499065</v>
       </c>
       <c r="H85" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$137:$M$137,$O$69:$V$69)*IF(Links!$E$137="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$137="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -34357,11 +34357,11 @@
       </c>
       <c r="I85" s="17" t="n">
         <f aca="false">G85-H85</f>
-        <v>-0.170310569937101</v>
+        <v>0</v>
       </c>
       <c r="J85" s="6" t="str">
         <f aca="false">IF(ROUND(G85-H85,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K85" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C85,Links!$B$218:$B$342,0)),1)</f>
@@ -34405,7 +34405,7 @@
       </c>
       <c r="G86" s="17" t="n">
         <f aca="false">INDEX(Links!$N$138:$W$138,1,(Resumen!$C$3-2025))</f>
-        <v>22.6283244618841</v>
+        <v>22.670394996375</v>
       </c>
       <c r="H86" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$138:$M$138,$O$69:$V$69)*IF(Links!$E$138="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$138="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -34413,7 +34413,7 @@
       </c>
       <c r="I86" s="17" t="n">
         <f aca="false">G86-H86</f>
-        <v>-0.0420705344908967</v>
+        <v>0</v>
       </c>
       <c r="J86" s="6" t="str">
         <f aca="false">IF(ROUND(G86-H86,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -34461,7 +34461,7 @@
       </c>
       <c r="G87" s="17" t="n">
         <f aca="false">INDEX(Links!$N$139:$W$139,1,(Resumen!$C$3-2025))</f>
-        <v>18.1427644650532</v>
+        <v>18.146821329</v>
       </c>
       <c r="H87" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$139:$M$139,$O$69:$V$69)*IF(Links!$E$139="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$139="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -34469,7 +34469,7 @@
       </c>
       <c r="I87" s="17" t="n">
         <f aca="false">G87-H87</f>
-        <v>-0.0040568639468006</v>
+        <v>0</v>
       </c>
       <c r="J87" s="6" t="str">
         <f aca="false">IF(ROUND(G87-H87,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -34517,7 +34517,7 @@
       </c>
       <c r="G88" s="17" t="n">
         <f aca="false">INDEX(Links!$N$140:$W$140,1,(Resumen!$C$3-2025))</f>
-        <v>7.7531911162633</v>
+        <v>7.76830533225</v>
       </c>
       <c r="H88" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$140:$M$140,$O$69:$V$69)*IF(Links!$E$140="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$140="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -34525,7 +34525,7 @@
       </c>
       <c r="I88" s="17" t="n">
         <f aca="false">G88-H88</f>
-        <v>-0.0151142159867002</v>
+        <v>0</v>
       </c>
       <c r="J88" s="6" t="str">
         <f aca="false">IF(ROUND(G88-H88,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -34573,7 +34573,7 @@
       </c>
       <c r="G89" s="17" t="n">
         <f aca="false">INDEX(Links!$N$141:$W$141,1,(Resumen!$C$3-2025))</f>
-        <v>775.2705332</v>
+        <v>777.3105332</v>
       </c>
       <c r="H89" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$141:$M$141,$O$69:$V$69)*IF(Links!$E$141="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$141="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -34581,11 +34581,11 @@
       </c>
       <c r="I89" s="17" t="n">
         <f aca="false">G89-H89</f>
-        <v>-2.03999999999996</v>
+        <v>0</v>
       </c>
       <c r="J89" s="6" t="str">
         <f aca="false">IF(ROUND(G89-H89,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K89" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C89,Links!$B$218:$B$342,0)),1)</f>
@@ -34629,7 +34629,7 @@
       </c>
       <c r="G90" s="17" t="n">
         <f aca="false">INDEX(Links!$N$142:$W$142,1,(Resumen!$C$3-2025))</f>
-        <v>1706.2599828204</v>
+        <v>1708.4351731</v>
       </c>
       <c r="H90" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$142:$M$142,$O$69:$V$69)*IF(Links!$E$142="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$142="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -34637,11 +34637,11 @@
       </c>
       <c r="I90" s="17" t="n">
         <f aca="false">G90-H90</f>
-        <v>-2.1751902796002</v>
+        <v>0</v>
       </c>
       <c r="J90" s="6" t="str">
         <f aca="false">IF(ROUND(G90-H90,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K90" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C90,Links!$B$218:$B$342,0)),1)</f>
@@ -34685,7 +34685,7 @@
       </c>
       <c r="G91" s="17" t="n">
         <f aca="false">INDEX(Links!$N$143:$W$143,1,(Resumen!$C$3-2025))</f>
-        <v>372.569856</v>
+        <v>374.129856</v>
       </c>
       <c r="H91" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$143:$M$143,$O$69:$V$69)*IF(Links!$E$143="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$143="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -34693,11 +34693,11 @@
       </c>
       <c r="I91" s="17" t="n">
         <f aca="false">G91-H91</f>
-        <v>-1.56</v>
+        <v>0</v>
       </c>
       <c r="J91" s="6" t="str">
         <f aca="false">IF(ROUND(G91-H91,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K91" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C91,Links!$B$218:$B$342,0)),1)</f>
@@ -34741,7 +34741,7 @@
       </c>
       <c r="G92" s="17" t="n">
         <f aca="false">INDEX(Links!$N$144:$W$144,1,(Resumen!$C$3-2025))</f>
-        <v>247.176074484914</v>
+        <v>247.4465706</v>
       </c>
       <c r="H92" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$144:$M$144,$O$69:$V$69)*IF(Links!$E$144="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$144="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -34749,11 +34749,11 @@
       </c>
       <c r="I92" s="17" t="n">
         <f aca="false">G92-H92</f>
-        <v>-0.270496115085962</v>
+        <v>0</v>
       </c>
       <c r="J92" s="6" t="str">
         <f aca="false">IF(ROUND(G92-H92,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K92" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C92,Links!$B$218:$B$342,0)),1)</f>
@@ -34797,7 +34797,7 @@
       </c>
       <c r="G93" s="17" t="n">
         <f aca="false">INDEX(Links!$N$145:$W$145,1,(Resumen!$C$3-2025))</f>
-        <v>91902.1824379067</v>
+        <v>91918.95765465</v>
       </c>
       <c r="H93" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$145:$M$145,$O$69:$V$69)*IF(Links!$E$145="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$145="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -34805,11 +34805,11 @@
       </c>
       <c r="I93" s="17" t="n">
         <f aca="false">G93-H93</f>
-        <v>-16.7752167433064</v>
+        <v>0</v>
       </c>
       <c r="J93" s="6" t="str">
         <f aca="false">IF(ROUND(G93-H93,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K93" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C93,Links!$B$218:$B$342,0)),1)</f>
@@ -34853,7 +34853,7 @@
       </c>
       <c r="G94" s="17" t="n">
         <f aca="false">INDEX(Links!$N$146:$W$146,1,(Resumen!$C$3-2025))</f>
-        <v>540.110594188926</v>
+        <v>540.223176538547</v>
       </c>
       <c r="H94" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$146:$M$146,$O$69:$V$69)*IF(Links!$E$146="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$146="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -34861,11 +34861,11 @@
       </c>
       <c r="I94" s="17" t="n">
         <f aca="false">G94-H94</f>
-        <v>-0.112582349620538</v>
+        <v>0</v>
       </c>
       <c r="J94" s="6" t="str">
         <f aca="false">IF(ROUND(G94-H94,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K94" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C94,Links!$B$218:$B$342,0)),1)</f>
@@ -34909,7 +34909,7 @@
       </c>
       <c r="G95" s="17" t="n">
         <f aca="false">INDEX(Links!$N$147:$W$147,1,(Resumen!$C$3-2025))</f>
-        <v>7257.10578602127</v>
+        <v>7258.7285316</v>
       </c>
       <c r="H95" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$147:$M$147,$O$69:$V$69)*IF(Links!$E$147="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$147="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -34917,11 +34917,11 @@
       </c>
       <c r="I95" s="17" t="n">
         <f aca="false">G95-H95</f>
-        <v>-1.62274557872934</v>
+        <v>0</v>
       </c>
       <c r="J95" s="6" t="str">
         <f aca="false">IF(ROUND(G95-H95,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K95" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C95,Links!$B$218:$B$342,0)),1)</f>
@@ -34965,7 +34965,7 @@
       </c>
       <c r="G96" s="17" t="n">
         <f aca="false">INDEX(Links!$N$148:$W$148,1,(Resumen!$C$3-2025))</f>
-        <v>3628.55289301064</v>
+        <v>3629.3642658</v>
       </c>
       <c r="H96" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$148:$M$148,$O$69:$V$69)*IF(Links!$E$148="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$148="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -34973,11 +34973,11 @@
       </c>
       <c r="I96" s="17" t="n">
         <f aca="false">G96-H96</f>
-        <v>-0.811372789359666</v>
+        <v>0</v>
       </c>
       <c r="J96" s="6" t="str">
         <f aca="false">IF(ROUND(G96-H96,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K96" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C96,Links!$B$218:$B$342,0)),1)</f>
@@ -35021,7 +35021,7 @@
       </c>
       <c r="G97" s="17" t="n">
         <f aca="false">INDEX(Links!$N$149:$W$149,1,(Resumen!$C$3-2025))</f>
-        <v>906.5410664</v>
+        <v>907.3410664</v>
       </c>
       <c r="H97" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$149:$M$149,$O$69:$V$69)*IF(Links!$E$149="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$149="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -35029,11 +35029,11 @@
       </c>
       <c r="I97" s="17" t="n">
         <f aca="false">G97-H97</f>
-        <v>-0.800000000000068</v>
+        <v>0</v>
       </c>
       <c r="J97" s="6" t="str">
         <f aca="false">IF(ROUND(G97-H97,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K97" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C97,Links!$B$218:$B$342,0)),1)</f>
@@ -35077,7 +35077,7 @@
       </c>
       <c r="G98" s="17" t="n">
         <f aca="false">INDEX(Links!$N$150:$W$150,1,(Resumen!$C$3-2025))</f>
-        <v>1996.51996564081</v>
+        <v>1995.9903462</v>
       </c>
       <c r="H98" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$150:$M$150,$O$69:$V$69)*IF(Links!$E$150="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$150="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -35085,7 +35085,7 @@
       </c>
       <c r="I98" s="17" t="n">
         <f aca="false">G98-H98</f>
-        <v>0.529619440809938</v>
+        <v>0</v>
       </c>
       <c r="J98" s="6" t="str">
         <f aca="false">IF(ROUND(G98-H98,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -35133,7 +35133,7 @@
       </c>
       <c r="G99" s="17" t="n">
         <f aca="false">INDEX(Links!$N$151:$W$151,1,(Resumen!$C$3-2025))</f>
-        <v>725.491860969828</v>
+        <v>726.0328532</v>
       </c>
       <c r="H99" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$151:$M$151,$O$69:$V$69)*IF(Links!$E$151="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$151="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -35141,11 +35141,11 @@
       </c>
       <c r="I99" s="17" t="n">
         <f aca="false">G99-H99</f>
-        <v>-0.540992230171923</v>
+        <v>0</v>
       </c>
       <c r="J99" s="6" t="str">
         <f aca="false">IF(ROUND(G99-H99,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K99" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C99,Links!$B$218:$B$342,0)),1)</f>
@@ -35189,7 +35189,7 @@
       </c>
       <c r="G100" s="17" t="n">
         <f aca="false">INDEX(Links!$N$152:$W$152,1,(Resumen!$C$3-2025))</f>
-        <v>453.2705332</v>
+        <v>453.6705332</v>
       </c>
       <c r="H100" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$152:$M$152,$O$69:$V$69)*IF(Links!$E$152="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$152="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -35197,11 +35197,11 @@
       </c>
       <c r="I100" s="17" t="n">
         <f aca="false">G100-H100</f>
-        <v>-0.400000000000034</v>
+        <v>0</v>
       </c>
       <c r="J100" s="6" t="str">
         <f aca="false">IF(ROUND(G100-H100,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K100" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C100,Links!$B$218:$B$342,0)),1)</f>
@@ -35245,7 +35245,7 @@
       </c>
       <c r="G101" s="17" t="n">
         <f aca="false">INDEX(Links!$N$153:$W$153,1,(Resumen!$C$3-2025))</f>
-        <v>1361.00591330532</v>
+        <v>1361.0115997</v>
       </c>
       <c r="H101" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$153:$M$153,$O$69:$V$69)*IF(Links!$E$153="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$153="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -35253,7 +35253,7 @@
       </c>
       <c r="I101" s="17" t="n">
         <f aca="false">G101-H101</f>
-        <v>-0.00568639467996945</v>
+        <v>0</v>
       </c>
       <c r="J101" s="6" t="str">
         <f aca="false">IF(ROUND(G101-H101,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -35301,7 +35301,7 @@
       </c>
       <c r="G102" s="17" t="n">
         <f aca="false">INDEX(Links!$N$154:$W$154,1,(Resumen!$C$3-2025))</f>
-        <v>1814.27644650532</v>
+        <v>1814.6821329</v>
       </c>
       <c r="H102" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$154:$M$154,$O$69:$V$69)*IF(Links!$E$154="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$154="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -35309,11 +35309,11 @@
       </c>
       <c r="I102" s="17" t="n">
         <f aca="false">G102-H102</f>
-        <v>-0.405686394679833</v>
+        <v>0</v>
       </c>
       <c r="J102" s="6" t="str">
         <f aca="false">IF(ROUND(G102-H102,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K102" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C102,Links!$B$218:$B$342,0)),1)</f>
@@ -35357,7 +35357,7 @@
       </c>
       <c r="G103" s="17" t="n">
         <f aca="false">INDEX(Links!$N$155:$W$155,1,(Resumen!$C$3-2025))</f>
-        <v>453.2705332</v>
+        <v>453.6705332</v>
       </c>
       <c r="H103" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$155:$M$155,$O$69:$V$69)*IF(Links!$E$155="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$155="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -35365,11 +35365,11 @@
       </c>
       <c r="I103" s="17" t="n">
         <f aca="false">G103-H103</f>
-        <v>-0.400000000000034</v>
+        <v>0</v>
       </c>
       <c r="J103" s="6" t="str">
         <f aca="false">IF(ROUND(G103-H103,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K103" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C103,Links!$B$218:$B$342,0)),1)</f>
@@ -35413,7 +35413,7 @@
       </c>
       <c r="G104" s="17" t="n">
         <f aca="false">INDEX(Links!$N$156:$W$156,1,(Resumen!$C$3-2025))</f>
-        <v>998.259982820404</v>
+        <v>997.9951731</v>
       </c>
       <c r="H104" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$156:$M$156,$O$69:$V$69)*IF(Links!$E$156="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$156="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -35421,7 +35421,7 @@
       </c>
       <c r="I104" s="17" t="n">
         <f aca="false">G104-H104</f>
-        <v>0.26480972040406</v>
+        <v>0</v>
       </c>
       <c r="J104" s="6" t="str">
         <f aca="false">IF(ROUND(G104-H104,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -35469,7 +35469,7 @@
       </c>
       <c r="G105" s="17" t="n">
         <f aca="false">INDEX(Links!$N$157:$W$157,1,(Resumen!$C$3-2025))</f>
-        <v>217.569856</v>
+        <v>217.809856</v>
       </c>
       <c r="H105" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$157:$M$157,$O$69:$V$69)*IF(Links!$E$157="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$157="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -35477,11 +35477,11 @@
       </c>
       <c r="I105" s="17" t="n">
         <f aca="false">G105-H105</f>
-        <v>-0.240000000000009</v>
+        <v>0</v>
       </c>
       <c r="J105" s="6" t="str">
         <f aca="false">IF(ROUND(G105-H105,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K105" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C105,Links!$B$218:$B$342,0)),1)</f>
@@ -35525,7 +35525,7 @@
       </c>
       <c r="G106" s="17" t="n">
         <f aca="false">INDEX(Links!$N$158:$W$158,1,(Resumen!$C$3-2025))</f>
-        <v>145.176074484914</v>
+        <v>145.2065706</v>
       </c>
       <c r="H106" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$158:$M$158,$O$69:$V$69)*IF(Links!$E$158="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$158="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -35533,7 +35533,7 @@
       </c>
       <c r="I106" s="17" t="n">
         <f aca="false">G106-H106</f>
-        <v>-0.030496115085981</v>
+        <v>0</v>
       </c>
       <c r="J106" s="6" t="str">
         <f aca="false">IF(ROUND(G106-H106,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -35581,7 +35581,7 @@
       </c>
       <c r="G107" s="17" t="n">
         <f aca="false">INDEX(Links!$N$159:$W$159,1,(Resumen!$C$3-2025))</f>
-        <v>453.2705332</v>
+        <v>453.6705332</v>
       </c>
       <c r="H107" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$159:$M$159,$O$69:$V$69)*IF(Links!$E$159="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$159="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -35589,11 +35589,11 @@
       </c>
       <c r="I107" s="17" t="n">
         <f aca="false">G107-H107</f>
-        <v>-0.400000000000034</v>
+        <v>0</v>
       </c>
       <c r="J107" s="6" t="str">
         <f aca="false">IF(ROUND(G107-H107,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K107" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C107,Links!$B$218:$B$342,0)),1)</f>
@@ -35637,7 +35637,7 @@
       </c>
       <c r="G108" s="17" t="n">
         <f aca="false">INDEX(Links!$N$160:$W$160,1,(Resumen!$C$3-2025))</f>
-        <v>998.259982820404</v>
+        <v>997.9951731</v>
       </c>
       <c r="H108" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$160:$M$160,$O$69:$V$69)*IF(Links!$E$160="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$160="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -35645,7 +35645,7 @@
       </c>
       <c r="I108" s="17" t="n">
         <f aca="false">G108-H108</f>
-        <v>0.26480972040406</v>
+        <v>0</v>
       </c>
       <c r="J108" s="6" t="str">
         <f aca="false">IF(ROUND(G108-H108,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -35693,7 +35693,7 @@
       </c>
       <c r="G109" s="17" t="n">
         <f aca="false">INDEX(Links!$N$161:$W$161,1,(Resumen!$C$3-2025))</f>
-        <v>217.569856</v>
+        <v>217.809856</v>
       </c>
       <c r="H109" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$161:$M$161,$O$69:$V$69)*IF(Links!$E$161="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$161="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -35701,11 +35701,11 @@
       </c>
       <c r="I109" s="17" t="n">
         <f aca="false">G109-H109</f>
-        <v>-0.240000000000009</v>
+        <v>0</v>
       </c>
       <c r="J109" s="6" t="str">
         <f aca="false">IF(ROUND(G109-H109,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K109" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C109,Links!$B$218:$B$342,0)),1)</f>
@@ -35749,7 +35749,7 @@
       </c>
       <c r="G110" s="17" t="n">
         <f aca="false">INDEX(Links!$N$162:$W$162,1,(Resumen!$C$3-2025))</f>
-        <v>145.176074484914</v>
+        <v>145.2065706</v>
       </c>
       <c r="H110" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$162:$M$162,$O$69:$V$69)*IF(Links!$E$162="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$162="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -35757,7 +35757,7 @@
       </c>
       <c r="I110" s="17" t="n">
         <f aca="false">G110-H110</f>
-        <v>-0.030496115085981</v>
+        <v>0</v>
       </c>
       <c r="J110" s="6" t="str">
         <f aca="false">IF(ROUND(G110-H110,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -35805,7 +35805,7 @@
       </c>
       <c r="G111" s="17" t="n">
         <f aca="false">INDEX(Links!$N$163:$W$163,1,(Resumen!$C$3-2025))</f>
-        <v>1451.5305160204</v>
+        <v>1451.6657063</v>
       </c>
       <c r="H111" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$163:$M$163,$O$69:$V$69)*IF(Links!$E$163="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$163="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -35813,11 +35813,11 @@
       </c>
       <c r="I111" s="17" t="n">
         <f aca="false">G111-H111</f>
-        <v>-0.13519027960001</v>
+        <v>0</v>
       </c>
       <c r="J111" s="6" t="str">
         <f aca="false">IF(ROUND(G111-H111,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K111" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C111,Links!$B$218:$B$342,0)),1)</f>
@@ -35861,7 +35861,7 @@
       </c>
       <c r="G112" s="17" t="n">
         <f aca="false">INDEX(Links!$N$164:$W$164,1,(Resumen!$C$3-2025))</f>
-        <v>362.745930484914</v>
+        <v>363.0164266</v>
       </c>
       <c r="H112" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$164:$M$164,$O$69:$V$69)*IF(Links!$E$164="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$164="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -35869,11 +35869,11 @@
       </c>
       <c r="I112" s="17" t="n">
         <f aca="false">G112-H112</f>
-        <v>-0.270496115085962</v>
+        <v>0</v>
       </c>
       <c r="J112" s="6" t="str">
         <f aca="false">IF(ROUND(G112-H112,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K112" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C112,Links!$B$218:$B$342,0)),1)</f>
@@ -35917,7 +35917,7 @@
       </c>
       <c r="G113" s="17" t="n">
         <f aca="false">INDEX(Links!$N$165:$W$165,1,(Resumen!$C$3-2025))</f>
-        <v>453.2705332</v>
+        <v>453.6705332</v>
       </c>
       <c r="H113" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$165:$M$165,$O$69:$V$69)*IF(Links!$E$165="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$165="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -35925,11 +35925,11 @@
       </c>
       <c r="I113" s="17" t="n">
         <f aca="false">G113-H113</f>
-        <v>-0.400000000000034</v>
+        <v>0</v>
       </c>
       <c r="J113" s="6" t="str">
         <f aca="false">IF(ROUND(G113-H113,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K113" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C113,Links!$B$218:$B$342,0)),1)</f>
@@ -35973,7 +35973,7 @@
       </c>
       <c r="G114" s="17" t="n">
         <f aca="false">INDEX(Links!$N$166:$W$166,1,(Resumen!$C$3-2025))</f>
-        <v>998.259982820404</v>
+        <v>997.9951731</v>
       </c>
       <c r="H114" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$166:$M$166,$O$69:$V$69)*IF(Links!$E$166="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$166="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -35981,7 +35981,7 @@
       </c>
       <c r="I114" s="17" t="n">
         <f aca="false">G114-H114</f>
-        <v>0.26480972040406</v>
+        <v>0</v>
       </c>
       <c r="J114" s="6" t="str">
         <f aca="false">IF(ROUND(G114-H114,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -36029,7 +36029,7 @@
       </c>
       <c r="G115" s="17" t="n">
         <f aca="false">INDEX(Links!$N$167:$W$167,1,(Resumen!$C$3-2025))</f>
-        <v>217.569856</v>
+        <v>217.809856</v>
       </c>
       <c r="H115" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$167:$M$167,$O$69:$V$69)*IF(Links!$E$167="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$167="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -36037,11 +36037,11 @@
       </c>
       <c r="I115" s="17" t="n">
         <f aca="false">G115-H115</f>
-        <v>-0.240000000000009</v>
+        <v>0</v>
       </c>
       <c r="J115" s="6" t="str">
         <f aca="false">IF(ROUND(G115-H115,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K115" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C115,Links!$B$218:$B$342,0)),1)</f>
@@ -36085,7 +36085,7 @@
       </c>
       <c r="G116" s="17" t="n">
         <f aca="false">INDEX(Links!$N$168:$W$168,1,(Resumen!$C$3-2025))</f>
-        <v>145.176074484914</v>
+        <v>145.2065706</v>
       </c>
       <c r="H116" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$168:$M$168,$O$69:$V$69)*IF(Links!$E$168="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$168="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -36093,7 +36093,7 @@
       </c>
       <c r="I116" s="17" t="n">
         <f aca="false">G116-H116</f>
-        <v>-0.030496115085981</v>
+        <v>0</v>
       </c>
       <c r="J116" s="6" t="str">
         <f aca="false">IF(ROUND(G116-H116,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -36141,7 +36141,7 @@
       </c>
       <c r="G117" s="17" t="n">
         <f aca="false">INDEX(Links!$N$169:$W$169,1,(Resumen!$C$3-2025))</f>
-        <v>1385.71683246007</v>
+        <v>1386.02668957523</v>
       </c>
       <c r="H117" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$169:$M$169,$O$69:$V$69)*IF(Links!$E$169="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$169="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -36149,11 +36149,11 @@
       </c>
       <c r="I117" s="17" t="n">
         <f aca="false">G117-H117</f>
-        <v>-0.309857115156774</v>
+        <v>0</v>
       </c>
       <c r="J117" s="6" t="str">
         <f aca="false">IF(ROUND(G117-H117,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K117" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C117,Links!$B$218:$B$342,0)),1)</f>
@@ -36197,7 +36197,7 @@
       </c>
       <c r="G118" s="17" t="n">
         <f aca="false">INDEX(Links!$N$170:$W$170,1,(Resumen!$C$3-2025))</f>
-        <v>1814.27644650532</v>
+        <v>1814.6821329</v>
       </c>
       <c r="H118" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$170:$M$170,$O$69:$V$69)*IF(Links!$E$170="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$170="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -36205,11 +36205,11 @@
       </c>
       <c r="I118" s="17" t="n">
         <f aca="false">G118-H118</f>
-        <v>-0.405686394679833</v>
+        <v>0</v>
       </c>
       <c r="J118" s="6" t="str">
         <f aca="false">IF(ROUND(G118-H118,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K118" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C118,Links!$B$218:$B$342,0)),1)</f>
@@ -36253,7 +36253,7 @@
       </c>
       <c r="G119" s="17" t="n">
         <f aca="false">INDEX(Links!$N$171:$W$171,1,(Resumen!$C$3-2025))</f>
-        <v>428.559614045248</v>
+        <v>428.655443324773</v>
       </c>
       <c r="H119" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$171:$M$171,$O$69:$V$69)*IF(Links!$E$171="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$171="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -36261,11 +36261,11 @@
       </c>
       <c r="I119" s="17" t="n">
         <f aca="false">G119-H119</f>
-        <v>-0.0958292795252191</v>
+        <v>0</v>
       </c>
       <c r="J119" s="6" t="str">
         <f aca="false">IF(ROUND(G119-H119,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K119" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C119,Links!$B$218:$B$342,0)),1)</f>
@@ -36309,7 +36309,7 @@
       </c>
       <c r="G120" s="17" t="n">
         <f aca="false">INDEX(Links!$N$172:$W$172,1,(Resumen!$C$3-2025))</f>
-        <v>1814.27644650532</v>
+        <v>1814.6821329</v>
       </c>
       <c r="H120" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$172:$M$172,$O$69:$V$69)*IF(Links!$E$172="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$172="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -36317,11 +36317,11 @@
       </c>
       <c r="I120" s="17" t="n">
         <f aca="false">G120-H120</f>
-        <v>-0.405686394679833</v>
+        <v>0</v>
       </c>
       <c r="J120" s="6" t="str">
         <f aca="false">IF(ROUND(G120-H120,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K120" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C120,Links!$B$218:$B$342,0)),1)</f>
@@ -36365,7 +36365,7 @@
       </c>
       <c r="G121" s="17" t="n">
         <f aca="false">INDEX(Links!$N$173:$W$173,1,(Resumen!$C$3-2025))</f>
-        <v>1814.27644650532</v>
+        <v>1814.6821329</v>
       </c>
       <c r="H121" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$173:$M$173,$O$69:$V$69)*IF(Links!$E$173="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$173="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -36373,11 +36373,11 @@
       </c>
       <c r="I121" s="17" t="n">
         <f aca="false">G121-H121</f>
-        <v>-0.405686394679833</v>
+        <v>0</v>
       </c>
       <c r="J121" s="6" t="str">
         <f aca="false">IF(ROUND(G121-H121,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K121" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C121,Links!$B$218:$B$342,0)),1)</f>
@@ -36421,7 +36421,7 @@
       </c>
       <c r="G122" s="17" t="n">
         <f aca="false">INDEX(Links!$N$174:$W$174,1,(Resumen!$C$3-2025))</f>
-        <v>1814.27644650532</v>
+        <v>1814.6821329</v>
       </c>
       <c r="H122" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$174:$M$174,$O$69:$V$69)*IF(Links!$E$174="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$174="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -36429,11 +36429,11 @@
       </c>
       <c r="I122" s="17" t="n">
         <f aca="false">G122-H122</f>
-        <v>-0.405686394679833</v>
+        <v>0</v>
       </c>
       <c r="J122" s="6" t="str">
         <f aca="false">IF(ROUND(G122-H122,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K122" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C122,Links!$B$218:$B$342,0)),1)</f>
@@ -36477,7 +36477,7 @@
       </c>
       <c r="G123" s="17" t="n">
         <f aca="false">INDEX(Links!$N$175:$W$175,1,(Resumen!$C$3-2025))</f>
-        <v>1287</v>
+        <v>1292.64</v>
       </c>
       <c r="H123" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$175:$M$175,$O$69:$V$69)*IF(Links!$E$175="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$175="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -36485,11 +36485,11 @@
       </c>
       <c r="I123" s="17" t="n">
         <f aca="false">G123-H123</f>
-        <v>-5.6400000000001</v>
+        <v>0</v>
       </c>
       <c r="J123" s="6" t="str">
         <f aca="false">IF(ROUND(G123-H123,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K123" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C123,Links!$B$218:$B$342,0)),1)</f>
@@ -36533,7 +36533,7 @@
       </c>
       <c r="G124" s="17" t="n">
         <f aca="false">INDEX(Links!$N$176:$W$176,1,(Resumen!$C$3-2025))</f>
-        <v>1030</v>
+        <v>1034.08</v>
       </c>
       <c r="H124" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$176:$M$176,$O$69:$V$69)*IF(Links!$E$176="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$176="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -36541,11 +36541,11 @@
       </c>
       <c r="I124" s="17" t="n">
         <f aca="false">G124-H124</f>
-        <v>-4.07999999999993</v>
+        <v>0</v>
       </c>
       <c r="J124" s="6" t="str">
         <f aca="false">IF(ROUND(G124-H124,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K124" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C124,Links!$B$218:$B$342,0)),1)</f>
@@ -36589,7 +36589,7 @@
       </c>
       <c r="G125" s="17" t="n">
         <f aca="false">INDEX(Links!$N$177:$W$177,1,(Resumen!$C$3-2025))</f>
-        <v>257</v>
+        <v>258.56</v>
       </c>
       <c r="H125" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$177:$M$177,$O$69:$V$69)*IF(Links!$E$177="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$177="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -36597,11 +36597,11 @@
       </c>
       <c r="I125" s="17" t="n">
         <f aca="false">G125-H125</f>
-        <v>-1.56</v>
+        <v>0</v>
       </c>
       <c r="J125" s="6" t="str">
         <f aca="false">IF(ROUND(G125-H125,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K125" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C125,Links!$B$218:$B$342,0)),1)</f>
@@ -36645,7 +36645,7 @@
       </c>
       <c r="G126" s="17" t="n">
         <f aca="false">INDEX(Links!$N$178:$W$178,1,(Resumen!$C$3-2025))</f>
-        <v>134.916666666667</v>
+        <v>135.516111111111</v>
       </c>
       <c r="H126" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$178:$M$178,$O$69:$V$69)*IF(Links!$E$178="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$178="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -36653,11 +36653,11 @@
       </c>
       <c r="I126" s="17" t="n">
         <f aca="false">G126-H126</f>
-        <v>-0.599444444444117</v>
+        <v>0</v>
       </c>
       <c r="J126" s="6" t="str">
         <f aca="false">IF(ROUND(G126-H126,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K126" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C126,Links!$B$218:$B$342,0)),1)</f>
@@ -36701,7 +36701,7 @@
       </c>
       <c r="G127" s="17" t="n">
         <f aca="false">INDEX(Links!$N$179:$W$179,1,(Resumen!$C$3-2025))</f>
-        <v>134.916666666667</v>
+        <v>135.516111111111</v>
       </c>
       <c r="H127" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$179:$M$179,$O$69:$V$69)*IF(Links!$E$179="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$179="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
@@ -36709,11 +36709,11 @@
       </c>
       <c r="I127" s="17" t="n">
         <f aca="false">G127-H127</f>
-        <v>-0.599444444444117</v>
+        <v>0</v>
       </c>
       <c r="J127" s="6" t="str">
         <f aca="false">IF(ROUND(G127-H127,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K127" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C127,Links!$B$218:$B$342,0)),1)</f>
@@ -36899,7 +36899,7 @@
       </c>
       <c r="G132" s="17" t="n">
         <f aca="false">INDEX(Links!$X$182:$AG$182,1,(Resumen!$C$3-2025))</f>
-        <v>42706.572139183</v>
+        <v>42315.769643171</v>
       </c>
       <c r="H132" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$182:$W$182,$O$130:$AF$130)*IF(Links!$E$182="CABA",INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),IF(Links!$E$182="PBA",1-INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),1))</f>
@@ -36907,7 +36907,7 @@
       </c>
       <c r="I132" s="17" t="n">
         <f aca="false">G132-H132</f>
-        <v>390.802496012009</v>
+        <v>0</v>
       </c>
       <c r="J132" s="6" t="str">
         <f aca="false">IF(ROUND(G132-H132,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -36955,7 +36955,7 @@
       </c>
       <c r="G133" s="17" t="n">
         <f aca="false">INDEX(Links!$X$183:$AG$183,1,(Resumen!$C$3-2025))</f>
-        <v>10553.0160608562</v>
+        <v>10613.9930281523</v>
       </c>
       <c r="H133" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$183:$W$183,$O$130:$AF$130)*IF(Links!$E$183="CABA",INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),IF(Links!$E$183="PBA",1-INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),1))</f>
@@ -36963,11 +36963,11 @@
       </c>
       <c r="I133" s="17" t="n">
         <f aca="false">G133-H133</f>
-        <v>-60.9769672960865</v>
+        <v>0</v>
       </c>
       <c r="J133" s="6" t="str">
         <f aca="false">IF(ROUND(G133-H133,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K133" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C133,Links!$B$218:$B$342,0)),1)</f>
@@ -37011,7 +37011,7 @@
       </c>
       <c r="G134" s="17" t="n">
         <f aca="false">INDEX(Links!$X$184:$AG$184,1,(Resumen!$C$3-2025))</f>
-        <v>725.457135307448</v>
+        <v>727.985233166422</v>
       </c>
       <c r="H134" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$184:$W$184,$O$130:$AF$130)*IF(Links!$E$184="CABA",INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),IF(Links!$E$184="PBA",1-INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),1))</f>
@@ -37019,11 +37019,11 @@
       </c>
       <c r="I134" s="17" t="n">
         <f aca="false">G134-H134</f>
-        <v>-2.52809785897387</v>
+        <v>0</v>
       </c>
       <c r="J134" s="6" t="str">
         <f aca="false">IF(ROUND(G134-H134,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K134" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C134,Links!$B$218:$B$342,0)),1)</f>
@@ -37067,7 +37067,7 @@
       </c>
       <c r="G135" s="17" t="n">
         <f aca="false">INDEX(Links!$X$185:$AG$185,1,(Resumen!$C$3-2025))</f>
-        <v>1163.06980253485</v>
+        <v>1170.00200918174</v>
       </c>
       <c r="H135" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$185:$W$185,$O$130:$AF$130)*IF(Links!$E$185="CABA",INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),IF(Links!$E$185="PBA",1-INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),1))</f>
@@ -37075,11 +37075,11 @@
       </c>
       <c r="I135" s="17" t="n">
         <f aca="false">G135-H135</f>
-        <v>-6.93220664688806</v>
+        <v>0</v>
       </c>
       <c r="J135" s="6" t="str">
         <f aca="false">IF(ROUND(G135-H135,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K135" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C135,Links!$B$218:$B$342,0)),1)</f>
@@ -37123,7 +37123,7 @@
       </c>
       <c r="G136" s="17" t="n">
         <f aca="false">INDEX(Links!$X$186:$AG$186,1,(Resumen!$C$3-2025))</f>
-        <v>2474.01024591012</v>
+        <v>2465.02054558444</v>
       </c>
       <c r="H136" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$186:$W$186,$O$130:$AF$130)*IF(Links!$E$186="CABA",INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),IF(Links!$E$186="PBA",1-INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),1))</f>
@@ -37131,7 +37131,7 @@
       </c>
       <c r="I136" s="17" t="n">
         <f aca="false">G136-H136</f>
-        <v>8.98970032568104</v>
+        <v>0</v>
       </c>
       <c r="J136" s="6" t="str">
         <f aca="false">IF(ROUND(G136-H136,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -37179,7 +37179,7 @@
       </c>
       <c r="G137" s="17" t="n">
         <f aca="false">INDEX(Links!$X$187:$AG$187,1,(Resumen!$C$3-2025))</f>
-        <v>185.038186767902</v>
+        <v>186.309928788795</v>
       </c>
       <c r="H137" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$187:$W$187,$O$130:$AF$130)*IF(Links!$E$187="CABA",INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),IF(Links!$E$187="PBA",1-INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),1))</f>
@@ -37187,11 +37187,11 @@
       </c>
       <c r="I137" s="17" t="n">
         <f aca="false">G137-H137</f>
-        <v>-1.27174202089299</v>
+        <v>0</v>
       </c>
       <c r="J137" s="6" t="str">
         <f aca="false">IF(ROUND(G137-H137,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K137" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C137,Links!$B$218:$B$342,0)),1)</f>
@@ -37235,7 +37235,7 @@
       </c>
       <c r="G138" s="17" t="n">
         <f aca="false">INDEX(Links!$X$188:$AG$188,1,(Resumen!$C$3-2025))</f>
-        <v>505.427368998169</v>
+        <v>506.637826734987</v>
       </c>
       <c r="H138" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$188:$W$188,$O$130:$AF$130)*IF(Links!$E$188="CABA",INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),IF(Links!$E$188="PBA",1-INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),1))</f>
@@ -37243,11 +37243,11 @@
       </c>
       <c r="I138" s="17" t="n">
         <f aca="false">G138-H138</f>
-        <v>-1.21045773681828</v>
+        <v>0</v>
       </c>
       <c r="J138" s="6" t="str">
         <f aca="false">IF(ROUND(G138-H138,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K138" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C138,Links!$B$218:$B$342,0)),1)</f>
@@ -37291,7 +37291,7 @@
       </c>
       <c r="G139" s="17" t="n">
         <f aca="false">INDEX(Links!$X$189:$AG$189,1,(Resumen!$C$3-2025))</f>
-        <v>7383.01305370899</v>
+        <v>7419.09878542082</v>
       </c>
       <c r="H139" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$189:$W$189,$O$130:$AF$130)*IF(Links!$E$189="CABA",INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),IF(Links!$E$189="PBA",1-INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),1))</f>
@@ -37299,11 +37299,11 @@
       </c>
       <c r="I139" s="17" t="n">
         <f aca="false">G139-H139</f>
-        <v>-36.0857317118262</v>
+        <v>0</v>
       </c>
       <c r="J139" s="6" t="str">
         <f aca="false">IF(ROUND(G139-H139,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K139" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C139,Links!$B$218:$B$342,0)),1)</f>
@@ -37347,7 +37347,7 @@
       </c>
       <c r="G140" s="17" t="n">
         <f aca="false">INDEX(Links!$X$190:$AG$190,1,(Resumen!$C$3-2025))</f>
-        <v>1852.60216272722</v>
+        <v>1843.53482815395</v>
       </c>
       <c r="H140" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$190:$W$190,$O$130:$AF$130)*IF(Links!$E$190="CABA",INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),IF(Links!$E$190="PBA",1-INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),1))</f>
@@ -37355,7 +37355,7 @@
       </c>
       <c r="I140" s="17" t="n">
         <f aca="false">G140-H140</f>
-        <v>9.06733457327437</v>
+        <v>0</v>
       </c>
       <c r="J140" s="6" t="str">
         <f aca="false">IF(ROUND(G140-H140,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -37403,7 +37403,7 @@
       </c>
       <c r="G141" s="17" t="n">
         <f aca="false">INDEX(Links!$X$191:$AG$191,1,(Resumen!$C$3-2025))</f>
-        <v>102177.896561299</v>
+        <v>101887.566999411</v>
       </c>
       <c r="H141" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$191:$W$191,$O$130:$AF$130)*IF(Links!$E$191="CABA",INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),IF(Links!$E$191="PBA",1-INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),1))</f>
@@ -37411,7 +37411,7 @@
       </c>
       <c r="I141" s="17" t="n">
         <f aca="false">G141-H141</f>
-        <v>290.329561887629</v>
+        <v>-3.63797880709171E-010</v>
       </c>
       <c r="J141" s="6" t="str">
         <f aca="false">IF(ROUND(G141-H141,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -37459,7 +37459,7 @@
       </c>
       <c r="G142" s="17" t="n">
         <f aca="false">INDEX(Links!$X$192:$AG$192,1,(Resumen!$C$3-2025))</f>
-        <v>3105.77010888421</v>
+        <v>3121.78618061568</v>
       </c>
       <c r="H142" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$192:$W$192,$O$130:$AF$130)*IF(Links!$E$192="CABA",INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),IF(Links!$E$192="PBA",1-INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),1))</f>
@@ -37467,11 +37467,11 @@
       </c>
       <c r="I142" s="17" t="n">
         <f aca="false">G142-H142</f>
-        <v>-16.0160717314729</v>
+        <v>0</v>
       </c>
       <c r="J142" s="6" t="str">
         <f aca="false">IF(ROUND(G142-H142,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K142" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C142,Links!$B$218:$B$342,0)),1)</f>
@@ -37515,7 +37515,7 @@
       </c>
       <c r="G143" s="17" t="n">
         <f aca="false">INDEX(Links!$X$193:$AG$193,1,(Resumen!$C$3-2025))</f>
-        <v>108186.304977739</v>
+        <v>107927.372813695</v>
       </c>
       <c r="H143" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$193:$W$193,$O$130:$AF$130)*IF(Links!$E$193="CABA",INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),IF(Links!$E$193="PBA",1-INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),1))</f>
@@ -37523,7 +37523,7 @@
       </c>
       <c r="I143" s="17" t="n">
         <f aca="false">G143-H143</f>
-        <v>258.932164044483</v>
+        <v>4.80213202536106E-010</v>
       </c>
       <c r="J143" s="6" t="str">
         <f aca="false">IF(ROUND(G143-H143,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -37571,7 +37571,7 @@
       </c>
       <c r="G144" s="17" t="n">
         <f aca="false">INDEX(Links!$X$194:$AG$194,1,(Resumen!$C$3-2025))</f>
-        <v>108186.304977739</v>
+        <v>107927.372813695</v>
       </c>
       <c r="H144" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$194:$W$194,$O$130:$AF$130)*IF(Links!$E$194="CABA",INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),IF(Links!$E$194="PBA",1-INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),1))</f>
@@ -37579,7 +37579,7 @@
       </c>
       <c r="I144" s="17" t="n">
         <f aca="false">G144-H144</f>
-        <v>258.932164044483</v>
+        <v>4.80213202536106E-010</v>
       </c>
       <c r="J144" s="6" t="str">
         <f aca="false">IF(ROUND(G144-H144,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -37627,7 +37627,7 @@
       </c>
       <c r="G145" s="17" t="n">
         <f aca="false">INDEX(Links!$X$195:$AG$195,1,(Resumen!$C$3-2025))</f>
-        <v>108186.304977739</v>
+        <v>107927.372813695</v>
       </c>
       <c r="H145" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$195:$W$195,$O$130:$AF$130)*IF(Links!$E$195="CABA",INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),IF(Links!$E$195="PBA",1-INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),1))</f>
@@ -37635,7 +37635,7 @@
       </c>
       <c r="I145" s="17" t="n">
         <f aca="false">G145-H145</f>
-        <v>258.932164044483</v>
+        <v>4.80213202536106E-010</v>
       </c>
       <c r="J145" s="6" t="str">
         <f aca="false">IF(ROUND(G145-H145,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -37683,7 +37683,7 @@
       </c>
       <c r="G146" s="17" t="n">
         <f aca="false">INDEX(Links!$X$196:$AG$196,1,(Resumen!$C$3-2025))</f>
-        <v>85734.5647571335</v>
+        <v>85529.3683934112</v>
       </c>
       <c r="H146" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$196:$W$196,$O$130:$AF$130)*IF(Links!$E$196="CABA",INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),IF(Links!$E$196="PBA",1-INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),1))</f>
@@ -37691,7 +37691,7 @@
       </c>
       <c r="I146" s="17" t="n">
         <f aca="false">G146-H146</f>
-        <v>205.196363722338</v>
+        <v>0</v>
       </c>
       <c r="J146" s="6" t="str">
         <f aca="false">IF(ROUND(G146-H146,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -37739,7 +37739,7 @@
       </c>
       <c r="G147" s="17" t="n">
         <f aca="false">INDEX(Links!$X$197:$AG$197,1,(Resumen!$C$3-2025))</f>
-        <v>85734.5647571335</v>
+        <v>85529.3683934112</v>
       </c>
       <c r="H147" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$197:$W$197,$O$130:$AF$130)*IF(Links!$E$197="CABA",INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),IF(Links!$E$197="PBA",1-INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),1))</f>
@@ -37747,7 +37747,7 @@
       </c>
       <c r="I147" s="17" t="n">
         <f aca="false">G147-H147</f>
-        <v>205.196363722338</v>
+        <v>0</v>
       </c>
       <c r="J147" s="6" t="str">
         <f aca="false">IF(ROUND(G147-H147,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -37795,7 +37795,7 @@
       </c>
       <c r="G148" s="17" t="n">
         <f aca="false">INDEX(Links!$X$198:$AG$198,1,(Resumen!$C$3-2025))</f>
-        <v>22451.7402206056</v>
+        <v>22398.0044202834</v>
       </c>
       <c r="H148" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$198:$W$198,$O$130:$AF$130)*IF(Links!$E$198="CABA",INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),IF(Links!$E$198="PBA",1-INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),1))</f>
@@ -37803,7 +37803,7 @@
       </c>
       <c r="I148" s="17" t="n">
         <f aca="false">G148-H148</f>
-        <v>53.735800322258</v>
+        <v>0</v>
       </c>
       <c r="J148" s="6" t="str">
         <f aca="false">IF(ROUND(G148-H148,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -37851,7 +37851,7 @@
       </c>
       <c r="G149" s="17" t="n">
         <f aca="false">INDEX(Links!$X$199:$AG$199,1,(Resumen!$C$3-2025))</f>
-        <v>278.050490711141</v>
+        <v>276.796497070763</v>
       </c>
       <c r="H149" s="17" t="n">
         <f aca="false">SUMPRODUCT(Links!$F$199:$W$199,$O$130:$AF$130)*IF(Links!$E$199="CABA",INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),IF(Links!$E$199="PBA",1-INDEX(Links!$C$14:$L$14,1,(Resumen!$C$3-2025)),1))</f>
@@ -37859,7 +37859,7 @@
       </c>
       <c r="I149" s="17" t="n">
         <f aca="false">G149-H149</f>
-        <v>1.2539936403777</v>
+        <v>0</v>
       </c>
       <c r="J149" s="6" t="str">
         <f aca="false">IF(ROUND(G149-H149,1)&gt;=0,"✔ Sí","✖ No")</f>
@@ -38240,7 +38240,7 @@
         <v>2908.13500312285</v>
       </c>
       <c r="H158" s="17" t="n">
-        <f aca="false">SUMPRODUCT(Links!$F$206:$N$206,$O$156:$W$156)*1</f>
+        <f aca="false">SUMPRODUCT(Links!$F$206:$N$206,$O$156:$W$156)*IF(Links!$E$206="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$206="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
         <v>2908.13500312285</v>
       </c>
       <c r="I158" s="17" t="n">
@@ -38296,7 +38296,7 @@
         <v>971.509933050576</v>
       </c>
       <c r="H159" s="17" t="n">
-        <f aca="false">SUMPRODUCT(Links!$F$207:$N$207,$O$156:$W$156)*1</f>
+        <f aca="false">SUMPRODUCT(Links!$F$207:$N$207,$O$156:$W$156)*IF(Links!$E$207="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$207="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
         <v>971.509933050576</v>
       </c>
       <c r="I159" s="17" t="n">
@@ -38352,7 +38352,7 @@
         <v>416.433346495834</v>
       </c>
       <c r="H160" s="17" t="n">
-        <f aca="false">SUMPRODUCT(Links!$F$208:$N$208,$O$156:$W$156)*1</f>
+        <f aca="false">SUMPRODUCT(Links!$F$208:$N$208,$O$156:$W$156)*IF(Links!$E$208="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$208="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
         <v>416.433346495834</v>
       </c>
       <c r="I160" s="17" t="n">
@@ -38408,7 +38408,7 @@
         <v>277.70377041365</v>
       </c>
       <c r="H161" s="17" t="n">
-        <f aca="false">SUMPRODUCT(Links!$F$209:$N$209,$O$156:$W$156)*1</f>
+        <f aca="false">SUMPRODUCT(Links!$F$209:$N$209,$O$156:$W$156)*IF(Links!$E$209="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$209="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
         <v>277.70377041365</v>
       </c>
       <c r="I161" s="17" t="n">
@@ -38464,7 +38464,7 @@
         <v>1650.60330969569</v>
       </c>
       <c r="H162" s="17" t="n">
-        <f aca="false">SUMPRODUCT(Links!$F$210:$N$210,$O$156:$W$156)*1</f>
+        <f aca="false">SUMPRODUCT(Links!$F$210:$N$210,$O$156:$W$156)*IF(Links!$E$210="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$210="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
         <v>1650.60330969569</v>
       </c>
       <c r="I162" s="17" t="n">
@@ -38520,7 +38520,7 @@
         <v>7005.27737</v>
       </c>
       <c r="H163" s="17" t="n">
-        <f aca="false">SUMPRODUCT(Links!$F$211:$N$211,$O$156:$W$156)*1</f>
+        <f aca="false">SUMPRODUCT(Links!$F$211:$N$211,$O$156:$W$156)*IF(Links!$E$211="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$211="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
         <v>7005.27737</v>
       </c>
       <c r="I163" s="17" t="n">
@@ -38576,7 +38576,7 @@
         <v>3776.01776725347</v>
       </c>
       <c r="H164" s="17" t="n">
-        <f aca="false">SUMPRODUCT(Links!$F$212:$N$212,$O$156:$W$156)*1</f>
+        <f aca="false">SUMPRODUCT(Links!$F$212:$N$212,$O$156:$W$156)*IF(Links!$E$212="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$212="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
         <v>3776.01776725347</v>
       </c>
       <c r="I164" s="17" t="n">
@@ -38632,7 +38632,7 @@
         <v>744.120454978018</v>
       </c>
       <c r="H165" s="17" t="n">
-        <f aca="false">SUMPRODUCT(Links!$F$213:$N$213,$O$156:$W$156)*1</f>
+        <f aca="false">SUMPRODUCT(Links!$F$213:$N$213,$O$156:$W$156)*IF(Links!$E$213="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$213="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
         <v>744.120454978018</v>
       </c>
       <c r="I165" s="17" t="n">
@@ -38688,7 +38688,7 @@
         <v>277.41598400273</v>
       </c>
       <c r="H166" s="17" t="n">
-        <f aca="false">SUMPRODUCT(Links!$F$214:$N$214,$O$156:$W$156)*1</f>
+        <f aca="false">SUMPRODUCT(Links!$F$214:$N$214,$O$156:$W$156)*IF(Links!$E$214="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$214="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
         <v>277.41598400273</v>
       </c>
       <c r="I166" s="17" t="n">
@@ -38744,16 +38744,16 @@
         <v>4258.3020622765</v>
       </c>
       <c r="H167" s="17" t="n">
-        <f aca="false">SUMPRODUCT(Links!$F$215:$N$215,$O$156:$W$156)*1</f>
-        <v>18027.2169390128</v>
+        <f aca="false">SUMPRODUCT(Links!$F$215:$N$215,$O$156:$W$156)*IF(Links!$E$215="CABA",INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),IF(Links!$E$215="PBA",1-INDEX(Links!$C$13:$L$13,1,(Resumen!$C$3-2025)),1))</f>
+        <v>4258.30206227651</v>
       </c>
       <c r="I167" s="17" t="n">
         <f aca="false">G167-H167</f>
-        <v>-13768.9148767363</v>
+        <v>0</v>
       </c>
       <c r="J167" s="6" t="str">
         <f aca="false">IF(ROUND(G167-H167,1)&gt;=0,"✔ Sí","✖ No")</f>
-        <v>✖ No</v>
+        <v>✔ Sí</v>
       </c>
       <c r="K167" s="17" t="n">
         <f aca="false">IFERROR(INDEX(Links!$C$345:$C$469,MATCH(C167,Links!$B$218:$B$342,0)),1)</f>
@@ -38761,7 +38761,7 @@
       </c>
       <c r="L167" s="17" t="n">
         <f aca="false">IF(K167&gt;0,H167/K167,0)</f>
-        <v>36.0544338780256</v>
+        <v>8.51660412455301</v>
       </c>
       <c r="M167" s="37" t="n">
         <f aca="false">IF(E167="kg",1,0)</f>

</xml_diff>

<commit_message>
Balanceo: marca al final de cada bloque IMPORTRANGE
Con los bloques vacíos, Google Sheets armaba Links hasta la última celda
con contenido (fila 2212) y las fórmulas que leen las últimas filas de
los bloques daban «La referencia no existe». Cada bloque lleva ahora una
celda ="" justo afuera de su esquina inferior derecha.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E33CYXtZ2f33D1RjoRdR65
</commit_message>
<xml_diff>
--- a/salida/Balanceo_Materiales_y_Linea.xlsx
+++ b/salida/Balanceo_Materiales_y_Linea.xlsx
@@ -1974,7 +1974,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:AG2219"/>
+  <dimension ref="A1:AH2220"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
@@ -2753,6 +2753,12 @@
       <c r="J58" s="8"/>
       <c r="K58" s="8"/>
       <c r="L58" s="8"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M59" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
@@ -3837,6 +3843,12 @@
       <c r="V120" s="9"/>
       <c r="W120" s="9"/>
     </row>
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="X121" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
+    </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="7" t="s">
         <v>18</v>
@@ -4872,6 +4884,12 @@
       <c r="U179" s="9"/>
       <c r="V179" s="9"/>
       <c r="W179" s="9"/>
+    </row>
+    <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="X180" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="7" t="s">
@@ -5389,6 +5407,12 @@
       <c r="AF203" s="9"/>
       <c r="AG203" s="9"/>
     </row>
+    <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="AH204" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
+    </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A205" s="7" t="s">
         <v>20</v>
@@ -5566,6 +5590,12 @@
       <c r="W215" s="9"/>
       <c r="X215" s="9"/>
     </row>
+    <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Y216" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
+    </row>
     <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A217" s="7" t="s">
         <v>21</v>
@@ -5949,6 +5979,12 @@
     <row r="342" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B342" s="10"/>
     </row>
+    <row r="343" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C343" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
+    </row>
     <row r="344" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A344" s="7" t="s">
         <v>22</v>
@@ -6456,6 +6492,12 @@
     <row r="469" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B469" s="10"/>
       <c r="C469" s="10"/>
+    </row>
+    <row r="470" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D470" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
     </row>
     <row r="471" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A471" s="7" t="s">
@@ -6740,6 +6782,12 @@
       <c r="I499" s="11"/>
       <c r="J499" s="11"/>
       <c r="K499" s="11"/>
+    </row>
+    <row r="500" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="L500" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
     </row>
     <row r="501" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A501" s="7" t="s">
@@ -8249,6 +8297,12 @@
       <c r="M610" s="11"/>
       <c r="N610" s="11"/>
     </row>
+    <row r="611" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O611" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
+    </row>
     <row r="612" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A612" s="7" t="s">
         <v>25</v>
@@ -8335,6 +8389,12 @@
     <row r="638" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B638" s="8"/>
     </row>
+    <row r="639" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C639" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
+    </row>
     <row r="640" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A640" s="7" t="s">
         <v>26</v>
@@ -8346,6 +8406,12 @@
         <v>150</v>
       </c>
     </row>
+    <row r="642" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C642" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
+    </row>
     <row r="643" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A643" s="7" t="s">
         <v>27</v>
@@ -9163,6 +9229,12 @@
     </row>
     <row r="922" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B922" s="11"/>
+    </row>
+    <row r="923" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C923" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
     </row>
     <row r="924" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A924" s="7" t="s">
@@ -10156,6 +10228,12 @@
       <c r="J1008" s="8"/>
       <c r="K1008" s="8"/>
     </row>
+    <row r="1009" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="L1009" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
+    </row>
     <row r="1010" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1010" s="7" t="s">
         <v>29</v>
@@ -10283,6 +10361,12 @@
       <c r="I1021" s="11"/>
       <c r="J1021" s="11"/>
       <c r="K1021" s="11"/>
+    </row>
+    <row r="1022" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="L1022" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
     </row>
     <row r="1023" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1023" s="7" t="s">
@@ -11792,6 +11876,12 @@
       <c r="M1132" s="11"/>
       <c r="N1132" s="11"/>
     </row>
+    <row r="1133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O1133" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
+    </row>
     <row r="1134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1134" s="7" t="s">
         <v>31</v>
@@ -11854,6 +11944,12 @@
     <row r="1152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1152" s="8"/>
     </row>
+    <row r="1153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C1153" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
+    </row>
     <row r="1154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1154" s="7" t="s">
         <v>32</v>
@@ -11865,6 +11961,12 @@
         <v>150</v>
       </c>
     </row>
+    <row r="1156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C1156" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
+    </row>
     <row r="1157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1157" s="7" t="s">
         <v>33</v>
@@ -12442,6 +12544,12 @@
     </row>
     <row r="1356" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1356" s="11"/>
+    </row>
+    <row r="1357" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C1357" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
     </row>
     <row r="1358" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1358" s="7" t="s">
@@ -13147,6 +13255,12 @@
       <c r="J1418" s="8"/>
       <c r="K1418" s="8"/>
     </row>
+    <row r="1419" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="L1419" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
+    </row>
     <row r="1420" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1420" s="7" t="s">
         <v>35</v>
@@ -13358,6 +13472,12 @@
       <c r="I1437" s="11"/>
       <c r="J1437" s="11"/>
       <c r="K1437" s="11"/>
+    </row>
+    <row r="1438" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="L1438" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
     </row>
     <row r="1439" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1439" s="7" t="s">
@@ -17717,6 +17837,12 @@
       <c r="M1757" s="11"/>
       <c r="N1757" s="11"/>
     </row>
+    <row r="1758" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O1758" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
+    </row>
     <row r="1759" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1759" s="7" t="s">
         <v>37</v>
@@ -17794,6 +17920,12 @@
     <row r="1782" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1782" s="12"/>
     </row>
+    <row r="1783" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C1783" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
+    </row>
     <row r="1784" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1784" s="7" t="s">
         <v>38</v>
@@ -17805,6 +17937,12 @@
         <v>150</v>
       </c>
     </row>
+    <row r="1786" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C1786" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
+    </row>
     <row r="1787" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1787" s="7" t="s">
         <v>39</v>
@@ -18532,6 +18670,12 @@
     </row>
     <row r="2099" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2099" s="11"/>
+    </row>
+    <row r="2100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C2100" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
     </row>
     <row r="2101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2101" s="7" t="s">
@@ -19417,6 +19561,12 @@
       <c r="J2188" s="8"/>
       <c r="K2188" s="8"/>
     </row>
+    <row r="2189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="L2189" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
+    </row>
     <row r="2190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2190" s="7" t="s">
         <v>41</v>
@@ -19524,6 +19674,12 @@
       <c r="I2199" s="13"/>
       <c r="J2199" s="13"/>
     </row>
+    <row r="2200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K2200" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
+    </row>
     <row r="2201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2201" s="7" t="s">
         <v>42</v>
@@ -19587,6 +19743,12 @@
       <c r="D2209" s="13"/>
       <c r="E2209" s="13"/>
       <c r="F2209" s="13"/>
+    </row>
+    <row r="2210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G2210" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
     </row>
     <row r="2211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2211" s="7" t="s">
@@ -19683,6 +19845,12 @@
       <c r="H2219" s="13"/>
       <c r="I2219" s="13"/>
       <c r="J2219" s="13"/>
+    </row>
+    <row r="2220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K2220" s="0" t="str">
+        <f aca="false">""</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="12">

</xml_diff>